<commit_message>
Updated spreadsheet again to fix equation on R10.
</commit_message>
<xml_diff>
--- a/Building A B Lighting New.xlsx
+++ b/Building A B Lighting New.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pacopoon/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E394EB1C-1ADD-1142-9D43-DE132B30826F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F31CB5C-A36D-7B42-966D-79C0DAF53044}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="25840" windowHeight="15300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -621,7 +621,7 @@
       <name val="Carlito"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -662,6 +662,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFF8FAFC"/>
         <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF8FBFD"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -740,7 +746,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -811,13 +817,17 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -826,6 +836,11 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FFF8FBFD"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -1007,29 +1022,29 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:24" ht="21">
-      <c r="A1" s="24" t="s">
+      <c r="A1" s="25" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
-      <c r="D1" s="24"/>
-      <c r="E1" s="24"/>
-      <c r="F1" s="24"/>
-      <c r="G1" s="24"/>
-      <c r="H1" s="24"/>
-      <c r="I1" s="24"/>
-      <c r="J1" s="24"/>
-      <c r="K1" s="24"/>
-      <c r="L1" s="24"/>
-      <c r="M1" s="24"/>
-      <c r="N1" s="24"/>
-      <c r="O1" s="24"/>
-      <c r="P1" s="24"/>
-      <c r="Q1" s="24"/>
-      <c r="R1" s="24"/>
-      <c r="S1" s="24"/>
-      <c r="T1" s="24"/>
-      <c r="U1" s="24"/>
+      <c r="B1" s="25"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
+      <c r="E1" s="25"/>
+      <c r="F1" s="25"/>
+      <c r="G1" s="25"/>
+      <c r="H1" s="25"/>
+      <c r="I1" s="25"/>
+      <c r="J1" s="25"/>
+      <c r="K1" s="25"/>
+      <c r="L1" s="25"/>
+      <c r="M1" s="25"/>
+      <c r="N1" s="25"/>
+      <c r="O1" s="25"/>
+      <c r="P1" s="25"/>
+      <c r="Q1" s="25"/>
+      <c r="R1" s="25"/>
+      <c r="S1" s="25"/>
+      <c r="T1" s="25"/>
+      <c r="U1" s="25"/>
     </row>
     <row r="2" spans="1:24" ht="48">
       <c r="A2" s="3" t="s">
@@ -1149,6 +1164,9 @@
       <c r="N3" s="20">
         <v>72</v>
       </c>
+      <c r="O3" s="27"/>
+      <c r="P3" s="27"/>
+      <c r="Q3" s="27"/>
       <c r="R3" s="20">
         <f>IF(OR(M3="",N3=""),"",M3*N3)</f>
         <v>72</v>
@@ -1163,7 +1181,7 @@
         <v/>
       </c>
       <c r="W3" s="20" t="str">
-        <f>IF(OR(R3="",V3=""),"",R3-V3)</f>
+        <f t="shared" ref="W3:W36" si="1">IF(OR(R3="",V3=""),"",R3-V3)</f>
         <v/>
       </c>
       <c r="X3" s="10" t="s">
@@ -1214,13 +1232,13 @@
       <c r="N4" s="20">
         <v>72</v>
       </c>
-      <c r="O4" s="9" t="s">
+      <c r="O4" s="28" t="s">
         <v>57</v>
       </c>
-      <c r="P4">
+      <c r="P4" s="27">
         <v>5</v>
       </c>
-      <c r="Q4">
+      <c r="Q4" s="27">
         <f>4*36</f>
         <v>144</v>
       </c>
@@ -1238,7 +1256,7 @@
         <v/>
       </c>
       <c r="W4" s="20" t="str">
-        <f>IF(OR(R4="",V4=""),"",R4-V4)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="X4" s="10" t="s">
@@ -1289,9 +1307,11 @@
       <c r="N5" s="20">
         <v>72</v>
       </c>
-      <c r="O5" s="9"/>
+      <c r="O5" s="28"/>
+      <c r="P5" s="27"/>
+      <c r="Q5" s="27"/>
       <c r="R5" s="20">
-        <f>IF(OR(M5="",N5=""),"",M5*N5)</f>
+        <f t="shared" ref="R5:R36" si="2">IF(OR(M5="",N5=""),"",M5*N5)</f>
         <v>72</v>
       </c>
       <c r="S5" s="9" t="s">
@@ -1300,11 +1320,11 @@
       <c r="T5" s="9"/>
       <c r="U5" s="20"/>
       <c r="V5" s="20" t="str">
-        <f t="shared" ref="V5:V36" si="1">IF(OR(T5="",U5=""),"",T5*U5)</f>
+        <f t="shared" ref="V5:V36" si="3">IF(OR(T5="",U5=""),"",T5*U5)</f>
         <v/>
       </c>
       <c r="W5" s="20" t="str">
-        <f>IF(OR(R5="",V5=""),"",R5-V5)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="X5" s="10" t="s">
@@ -1355,8 +1375,11 @@
       <c r="N6" s="20">
         <v>72</v>
       </c>
+      <c r="O6" s="27"/>
+      <c r="P6" s="27"/>
+      <c r="Q6" s="27"/>
       <c r="R6" s="20">
-        <f>IF(OR(M6="",N6=""),"",M6*N6)</f>
+        <f t="shared" si="2"/>
         <v>72</v>
       </c>
       <c r="S6" s="9" t="s">
@@ -1365,11 +1388,11 @@
       <c r="T6" s="9"/>
       <c r="U6" s="20"/>
       <c r="V6" s="20" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="W6" s="20" t="str">
-        <f>IF(OR(R6="",V6=""),"",R6-V6)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="X6" s="10" t="s">
@@ -1420,8 +1443,11 @@
       <c r="N7" s="20">
         <v>72</v>
       </c>
+      <c r="O7" s="27"/>
+      <c r="P7" s="27"/>
+      <c r="Q7" s="27"/>
       <c r="R7" s="20">
-        <f>IF(OR(M7="",N7=""),"",M7*N7)</f>
+        <f t="shared" si="2"/>
         <v>72</v>
       </c>
       <c r="S7" s="9" t="s">
@@ -1430,11 +1456,11 @@
       <c r="T7" s="9"/>
       <c r="U7" s="20"/>
       <c r="V7" s="20" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="W7" s="20" t="str">
-        <f>IF(OR(R7="",V7=""),"",R7-V7)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="X7" s="10" t="s">
@@ -1485,8 +1511,11 @@
       <c r="N8" s="20">
         <v>144</v>
       </c>
+      <c r="O8" s="27"/>
+      <c r="P8" s="27"/>
+      <c r="Q8" s="27"/>
       <c r="R8" s="20">
-        <f>IF(OR(M8="",N8=""),"",M8*N8)</f>
+        <f t="shared" si="2"/>
         <v>288</v>
       </c>
       <c r="S8" s="9" t="s">
@@ -1495,11 +1524,11 @@
       <c r="T8" s="9"/>
       <c r="U8" s="20"/>
       <c r="V8" s="20" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="W8" s="20" t="str">
-        <f>IF(OR(R8="",V8=""),"",R8-V8)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="X8" s="10" t="s">
@@ -1550,8 +1579,11 @@
       <c r="N9" s="20">
         <v>144</v>
       </c>
+      <c r="O9" s="27"/>
+      <c r="P9" s="27"/>
+      <c r="Q9" s="27"/>
       <c r="R9" s="20">
-        <f>IF(OR(M9="",N9=""),"",M9*N9)</f>
+        <f t="shared" si="2"/>
         <v>288</v>
       </c>
       <c r="S9" s="9" t="s">
@@ -1560,11 +1592,11 @@
       <c r="T9" s="9"/>
       <c r="U9" s="20"/>
       <c r="V9" s="20" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="W9" s="20" t="str">
-        <f>IF(OR(R9="",V9=""),"",R9-V9)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="X9" s="10" t="s">
@@ -1615,19 +1647,19 @@
       <c r="N10" s="20">
         <v>72</v>
       </c>
-      <c r="O10" s="9" t="s">
+      <c r="O10" s="28" t="s">
         <v>57</v>
       </c>
-      <c r="P10">
+      <c r="P10" s="27">
         <v>4</v>
       </c>
-      <c r="Q10">
+      <c r="Q10" s="27">
         <f>4*36</f>
         <v>144</v>
       </c>
       <c r="R10" s="20">
-        <f>IF(OR(M10="",N10=""),"",M10*N10)</f>
-        <v>288</v>
+        <f>IF(OR(M10="",N10=""),"",M10*N10+Q10)</f>
+        <v>432</v>
       </c>
       <c r="S10" s="9" t="s">
         <v>31</v>
@@ -1635,11 +1667,11 @@
       <c r="T10" s="9"/>
       <c r="U10" s="20"/>
       <c r="V10" s="20" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="W10" s="20" t="str">
-        <f>IF(OR(R10="",V10=""),"",R10-V10)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="X10" s="10" t="s">
@@ -1690,8 +1722,11 @@
       <c r="N11" s="20">
         <v>144</v>
       </c>
+      <c r="O11" s="27"/>
+      <c r="P11" s="27"/>
+      <c r="Q11" s="27"/>
       <c r="R11" s="20">
-        <f>IF(OR(M11="",N11=""),"",M11*N11)</f>
+        <f t="shared" si="2"/>
         <v>288</v>
       </c>
       <c r="S11" s="9" t="s">
@@ -1700,11 +1735,11 @@
       <c r="T11" s="9"/>
       <c r="U11" s="20"/>
       <c r="V11" s="20" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="W11" s="20" t="str">
-        <f>IF(OR(R11="",V11=""),"",R11-V11)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="X11" s="10" t="s">
@@ -1755,8 +1790,11 @@
       <c r="N12" s="20">
         <v>144</v>
       </c>
+      <c r="O12" s="27"/>
+      <c r="P12" s="27"/>
+      <c r="Q12" s="27"/>
       <c r="R12" s="20">
-        <f>IF(OR(M12="",N12=""),"",M12*N12)</f>
+        <f t="shared" si="2"/>
         <v>576</v>
       </c>
       <c r="S12" s="9" t="s">
@@ -1765,11 +1803,11 @@
       <c r="T12" s="9"/>
       <c r="U12" s="20"/>
       <c r="V12" s="20" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="W12" s="20" t="str">
-        <f>IF(OR(R12="",V12=""),"",R12-V12)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="X12" s="10" t="s">
@@ -1820,8 +1858,11 @@
       <c r="N13" s="20">
         <v>144</v>
       </c>
+      <c r="O13" s="27"/>
+      <c r="P13" s="27"/>
+      <c r="Q13" s="27"/>
       <c r="R13" s="20">
-        <f>IF(OR(M13="",N13=""),"",M13*N13)</f>
+        <f t="shared" si="2"/>
         <v>576</v>
       </c>
       <c r="S13" s="9" t="s">
@@ -1830,11 +1871,11 @@
       <c r="T13" s="9"/>
       <c r="U13" s="20"/>
       <c r="V13" s="20" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="W13" s="20" t="str">
-        <f>IF(OR(R13="",V13=""),"",R13-V13)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="X13" s="10" t="s">
@@ -1885,8 +1926,11 @@
       <c r="N14" s="20">
         <v>144</v>
       </c>
+      <c r="O14" s="27"/>
+      <c r="P14" s="27"/>
+      <c r="Q14" s="27"/>
       <c r="R14" s="20">
-        <f>IF(OR(M14="",N14=""),"",M14*N14)</f>
+        <f t="shared" si="2"/>
         <v>864</v>
       </c>
       <c r="S14" s="9" t="s">
@@ -1895,11 +1939,11 @@
       <c r="T14" s="9"/>
       <c r="U14" s="20"/>
       <c r="V14" s="20" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="W14" s="20" t="str">
-        <f>IF(OR(R14="",V14=""),"",R14-V14)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="X14" s="10" t="s">
@@ -1950,8 +1994,11 @@
       <c r="N15" s="20">
         <v>144</v>
       </c>
+      <c r="O15" s="27"/>
+      <c r="P15" s="27"/>
+      <c r="Q15" s="27"/>
       <c r="R15" s="20">
-        <f>IF(OR(M15="",N15=""),"",M15*N15)</f>
+        <f t="shared" si="2"/>
         <v>432</v>
       </c>
       <c r="S15" s="9" t="s">
@@ -1960,11 +2007,11 @@
       <c r="T15" s="9"/>
       <c r="U15" s="20"/>
       <c r="V15" s="20" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="W15" s="20" t="str">
-        <f>IF(OR(R15="",V15=""),"",R15-V15)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="X15" s="10" t="s">
@@ -2015,8 +2062,11 @@
       <c r="N16" s="20">
         <v>144</v>
       </c>
+      <c r="O16" s="27"/>
+      <c r="P16" s="27"/>
+      <c r="Q16" s="27"/>
       <c r="R16" s="20">
-        <f>IF(OR(M16="",N16=""),"",M16*N16)</f>
+        <f t="shared" si="2"/>
         <v>432</v>
       </c>
       <c r="S16" s="9" t="s">
@@ -2025,11 +2075,11 @@
       <c r="T16" s="9"/>
       <c r="U16" s="20"/>
       <c r="V16" s="20" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="W16" s="20" t="str">
-        <f>IF(OR(R16="",V16=""),"",R16-V16)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="X16" s="10" t="s">
@@ -2080,8 +2130,11 @@
       <c r="N17" s="20">
         <v>72</v>
       </c>
+      <c r="O17" s="27"/>
+      <c r="P17" s="27"/>
+      <c r="Q17" s="27"/>
       <c r="R17" s="20">
-        <f>IF(OR(M17="",N17=""),"",M17*N17)</f>
+        <f t="shared" si="2"/>
         <v>72</v>
       </c>
       <c r="S17" s="9" t="s">
@@ -2090,11 +2143,11 @@
       <c r="T17" s="9"/>
       <c r="U17" s="20"/>
       <c r="V17" s="20" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="W17" s="20" t="str">
-        <f>IF(OR(R17="",V17=""),"",R17-V17)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="X17" s="10" t="s">
@@ -2145,8 +2198,11 @@
       <c r="N18" s="20">
         <v>72</v>
       </c>
+      <c r="O18" s="27"/>
+      <c r="P18" s="27"/>
+      <c r="Q18" s="27"/>
       <c r="R18" s="20">
-        <f>IF(OR(M18="",N18=""),"",M18*N18)</f>
+        <f t="shared" si="2"/>
         <v>288</v>
       </c>
       <c r="S18" s="9" t="s">
@@ -2155,11 +2211,11 @@
       <c r="T18" s="9"/>
       <c r="U18" s="20"/>
       <c r="V18" s="20" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="W18" s="20" t="str">
-        <f>IF(OR(R18="",V18=""),"",R18-V18)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="X18" s="10" t="s">
@@ -2210,8 +2266,11 @@
       <c r="N19" s="20">
         <v>144</v>
       </c>
+      <c r="O19" s="27"/>
+      <c r="P19" s="27"/>
+      <c r="Q19" s="27"/>
       <c r="R19" s="20">
-        <f>IF(OR(M19="",N19=""),"",M19*N19)</f>
+        <f t="shared" si="2"/>
         <v>288</v>
       </c>
       <c r="S19" s="9" t="s">
@@ -2220,11 +2279,11 @@
       <c r="T19" s="9"/>
       <c r="U19" s="20"/>
       <c r="V19" s="20" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="W19" s="20" t="str">
-        <f>IF(OR(R19="",V19=""),"",R19-V19)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="X19" s="10" t="s">
@@ -2275,8 +2334,11 @@
       <c r="N20" s="20">
         <v>144</v>
       </c>
+      <c r="O20" s="27"/>
+      <c r="P20" s="27"/>
+      <c r="Q20" s="27"/>
       <c r="R20" s="20">
-        <f>IF(OR(M20="",N20=""),"",M20*N20)</f>
+        <f t="shared" si="2"/>
         <v>1008</v>
       </c>
       <c r="S20" s="9" t="s">
@@ -2285,11 +2347,11 @@
       <c r="T20" s="9"/>
       <c r="U20" s="20"/>
       <c r="V20" s="20" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="W20" s="20" t="str">
-        <f>IF(OR(R20="",V20=""),"",R20-V20)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="X20" s="10" t="s">
@@ -2340,8 +2402,11 @@
       <c r="N21" s="20">
         <v>72</v>
       </c>
+      <c r="O21" s="27"/>
+      <c r="P21" s="27"/>
+      <c r="Q21" s="27"/>
       <c r="R21" s="20">
-        <f>IF(OR(M21="",N21=""),"",M21*N21)</f>
+        <f t="shared" si="2"/>
         <v>72</v>
       </c>
       <c r="S21" s="9" t="s">
@@ -2350,11 +2415,11 @@
       <c r="T21" s="9"/>
       <c r="U21" s="20"/>
       <c r="V21" s="20" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="W21" s="20" t="str">
-        <f>IF(OR(R21="",V21=""),"",R21-V21)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="X21" s="10" t="s">
@@ -2405,8 +2470,11 @@
       <c r="N22" s="20">
         <v>72</v>
       </c>
+      <c r="O22" s="27"/>
+      <c r="P22" s="27"/>
+      <c r="Q22" s="27"/>
       <c r="R22" s="20">
-        <f>IF(OR(M22="",N22=""),"",M22*N22)</f>
+        <f t="shared" si="2"/>
         <v>144</v>
       </c>
       <c r="S22" s="9" t="s">
@@ -2415,11 +2483,11 @@
       <c r="T22" s="9"/>
       <c r="U22" s="20"/>
       <c r="V22" s="20" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="W22" s="20" t="str">
-        <f>IF(OR(R22="",V22=""),"",R22-V22)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="X22" s="10" t="s">
@@ -2461,7 +2529,7 @@
       <c r="K23" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="L23" s="26" t="s">
+      <c r="L23" s="24" t="s">
         <v>30</v>
       </c>
       <c r="M23" s="9">
@@ -2470,8 +2538,11 @@
       <c r="N23" s="20">
         <v>144</v>
       </c>
+      <c r="O23" s="27"/>
+      <c r="P23" s="27"/>
+      <c r="Q23" s="27"/>
       <c r="R23" s="20">
-        <f>IF(OR(M23="",N23=""),"",M23*N23)</f>
+        <f t="shared" si="2"/>
         <v>864</v>
       </c>
       <c r="S23" s="9" t="s">
@@ -2480,11 +2551,11 @@
       <c r="T23" s="9"/>
       <c r="U23" s="20"/>
       <c r="V23" s="20" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="W23" s="20" t="str">
-        <f>IF(OR(R23="",V23=""),"",R23-V23)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="X23" s="10" t="s">
@@ -2526,7 +2597,7 @@
       <c r="K24" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="L24" s="26" t="s">
+      <c r="L24" s="24" t="s">
         <v>30</v>
       </c>
       <c r="M24" s="9">
@@ -2535,8 +2606,11 @@
       <c r="N24" s="20">
         <v>144</v>
       </c>
+      <c r="O24" s="27"/>
+      <c r="P24" s="27"/>
+      <c r="Q24" s="27"/>
       <c r="R24" s="20">
-        <f>IF(OR(M24="",N24=""),"",M24*N24)</f>
+        <f t="shared" si="2"/>
         <v>576</v>
       </c>
       <c r="S24" s="9" t="s">
@@ -2545,11 +2619,11 @@
       <c r="T24" s="9"/>
       <c r="U24" s="20"/>
       <c r="V24" s="20" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="W24" s="20" t="str">
-        <f>IF(OR(R24="",V24=""),"",R24-V24)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="X24" s="10" t="s">
@@ -2591,7 +2665,7 @@
       <c r="K25" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="L25" s="26" t="s">
+      <c r="L25" s="24" t="s">
         <v>30</v>
       </c>
       <c r="M25" s="9">
@@ -2600,8 +2674,11 @@
       <c r="N25" s="20">
         <v>144</v>
       </c>
+      <c r="O25" s="27"/>
+      <c r="P25" s="27"/>
+      <c r="Q25" s="27"/>
       <c r="R25" s="20">
-        <f>IF(OR(M25="",N25=""),"",M25*N25)</f>
+        <f t="shared" si="2"/>
         <v>576</v>
       </c>
       <c r="S25" s="9" t="s">
@@ -2610,11 +2687,11 @@
       <c r="T25" s="9"/>
       <c r="U25" s="20"/>
       <c r="V25" s="20" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="W25" s="20" t="str">
-        <f>IF(OR(R25="",V25=""),"",R25-V25)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="X25" s="10" t="s">
@@ -2656,7 +2733,7 @@
       <c r="K26" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="L26" s="26" t="s">
+      <c r="L26" s="24" t="s">
         <v>30</v>
       </c>
       <c r="M26" s="9">
@@ -2665,8 +2742,11 @@
       <c r="N26" s="20">
         <v>144</v>
       </c>
+      <c r="O26" s="27"/>
+      <c r="P26" s="27"/>
+      <c r="Q26" s="27"/>
       <c r="R26" s="20">
-        <f>IF(OR(M26="",N26=""),"",M26*N26)</f>
+        <f t="shared" si="2"/>
         <v>1152</v>
       </c>
       <c r="S26" s="9" t="s">
@@ -2675,11 +2755,11 @@
       <c r="T26" s="9"/>
       <c r="U26" s="20"/>
       <c r="V26" s="20" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="W26" s="20" t="str">
-        <f>IF(OR(R26="",V26=""),"",R26-V26)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="X26" s="10" t="s">
@@ -2730,8 +2810,11 @@
       <c r="N27" s="20">
         <v>72</v>
       </c>
+      <c r="O27" s="27"/>
+      <c r="P27" s="27"/>
+      <c r="Q27" s="27"/>
       <c r="R27" s="20">
-        <f>IF(OR(M27="",N27=""),"",M27*N27)</f>
+        <f t="shared" si="2"/>
         <v>576</v>
       </c>
       <c r="S27" s="9" t="s">
@@ -2740,11 +2823,11 @@
       <c r="T27" s="9"/>
       <c r="U27" s="20"/>
       <c r="V27" s="20" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="W27" s="20" t="str">
-        <f>IF(OR(R27="",V27=""),"",R27-V27)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="X27" s="10" t="s">
@@ -2786,7 +2869,7 @@
       <c r="K28" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="L28" s="26" t="s">
+      <c r="L28" s="24" t="s">
         <v>30</v>
       </c>
       <c r="M28" s="9">
@@ -2795,8 +2878,11 @@
       <c r="N28" s="20">
         <v>144</v>
       </c>
+      <c r="O28" s="27"/>
+      <c r="P28" s="27"/>
+      <c r="Q28" s="27"/>
       <c r="R28" s="20">
-        <f>IF(OR(M28="",N28=""),"",M28*N28)</f>
+        <f t="shared" si="2"/>
         <v>1152</v>
       </c>
       <c r="S28" s="9" t="s">
@@ -2805,11 +2891,11 @@
       <c r="T28" s="9"/>
       <c r="U28" s="20"/>
       <c r="V28" s="20" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="W28" s="20" t="str">
-        <f>IF(OR(R28="",V28=""),"",R28-V28)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="X28" s="10" t="s">
@@ -2860,8 +2946,11 @@
       <c r="N29" s="20">
         <v>72</v>
       </c>
+      <c r="O29" s="27"/>
+      <c r="P29" s="27"/>
+      <c r="Q29" s="27"/>
       <c r="R29" s="20">
-        <f>IF(OR(M29="",N29=""),"",M29*N29)</f>
+        <f t="shared" si="2"/>
         <v>72</v>
       </c>
       <c r="S29" s="9" t="s">
@@ -2870,11 +2959,11 @@
       <c r="T29" s="9"/>
       <c r="U29" s="20"/>
       <c r="V29" s="20" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="W29" s="20" t="str">
-        <f>IF(OR(R29="",V29=""),"",R29-V29)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="X29" s="10" t="s">
@@ -2916,7 +3005,7 @@
       <c r="K30" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="L30" s="26" t="s">
+      <c r="L30" s="24" t="s">
         <v>30</v>
       </c>
       <c r="M30" s="9">
@@ -2925,8 +3014,11 @@
       <c r="N30" s="20">
         <v>144</v>
       </c>
+      <c r="O30" s="27"/>
+      <c r="P30" s="27"/>
+      <c r="Q30" s="27"/>
       <c r="R30" s="20">
-        <f>IF(OR(M30="",N30=""),"",M30*N30)</f>
+        <f t="shared" si="2"/>
         <v>576</v>
       </c>
       <c r="S30" s="9" t="s">
@@ -2935,11 +3027,11 @@
       <c r="T30" s="9"/>
       <c r="U30" s="20"/>
       <c r="V30" s="20" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="W30" s="20" t="str">
-        <f>IF(OR(R30="",V30=""),"",R30-V30)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="X30" s="10" t="s">
@@ -2981,7 +3073,7 @@
       <c r="K31" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="L31" s="26" t="s">
+      <c r="L31" s="24" t="s">
         <v>30</v>
       </c>
       <c r="M31" s="9">
@@ -2990,8 +3082,11 @@
       <c r="N31" s="20">
         <v>144</v>
       </c>
+      <c r="O31" s="27"/>
+      <c r="P31" s="27"/>
+      <c r="Q31" s="27"/>
       <c r="R31" s="20">
-        <f>IF(OR(M31="",N31=""),"",M31*N31)</f>
+        <f t="shared" si="2"/>
         <v>576</v>
       </c>
       <c r="S31" s="9" t="s">
@@ -3000,11 +3095,11 @@
       <c r="T31" s="9"/>
       <c r="U31" s="20"/>
       <c r="V31" s="20" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="W31" s="20" t="str">
-        <f>IF(OR(R31="",V31=""),"",R31-V31)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="X31" s="10" t="s">
@@ -3046,7 +3141,7 @@
       <c r="K32" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="L32" s="26" t="s">
+      <c r="L32" s="24" t="s">
         <v>30</v>
       </c>
       <c r="M32" s="9">
@@ -3055,8 +3150,11 @@
       <c r="N32" s="20">
         <v>144</v>
       </c>
+      <c r="O32" s="27"/>
+      <c r="P32" s="27"/>
+      <c r="Q32" s="27"/>
       <c r="R32" s="20">
-        <f>IF(OR(M32="",N32=""),"",M32*N32)</f>
+        <f t="shared" si="2"/>
         <v>576</v>
       </c>
       <c r="S32" s="9" t="s">
@@ -3065,11 +3163,11 @@
       <c r="T32" s="9"/>
       <c r="U32" s="20"/>
       <c r="V32" s="20" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="W32" s="20" t="str">
-        <f>IF(OR(R32="",V32=""),"",R32-V32)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="X32" s="10" t="s">
@@ -3120,8 +3218,11 @@
       <c r="N33" s="20">
         <v>72</v>
       </c>
+      <c r="O33" s="27"/>
+      <c r="P33" s="27"/>
+      <c r="Q33" s="27"/>
       <c r="R33" s="20">
-        <f>IF(OR(M33="",N33=""),"",M33*N33)</f>
+        <f t="shared" si="2"/>
         <v>72</v>
       </c>
       <c r="S33" s="9" t="s">
@@ -3130,11 +3231,11 @@
       <c r="T33" s="9"/>
       <c r="U33" s="20"/>
       <c r="V33" s="20" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="W33" s="20" t="str">
-        <f>IF(OR(R33="",V33=""),"",R33-V33)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="X33" s="10" t="s">
@@ -3185,8 +3286,11 @@
       <c r="N34" s="20">
         <v>72</v>
       </c>
+      <c r="O34" s="27"/>
+      <c r="P34" s="27"/>
+      <c r="Q34" s="27"/>
       <c r="R34" s="20">
-        <f>IF(OR(M34="",N34=""),"",M34*N34)</f>
+        <f t="shared" si="2"/>
         <v>72</v>
       </c>
       <c r="S34" s="9" t="s">
@@ -3195,11 +3299,11 @@
       <c r="T34" s="9"/>
       <c r="U34" s="20"/>
       <c r="V34" s="20" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="W34" s="20" t="str">
-        <f>IF(OR(R34="",V34=""),"",R34-V34)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="X34" s="10" t="s">
@@ -3241,7 +3345,7 @@
       <c r="K35" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="L35" s="26" t="s">
+      <c r="L35" s="24" t="s">
         <v>30</v>
       </c>
       <c r="M35" s="9">
@@ -3250,8 +3354,11 @@
       <c r="N35" s="20">
         <v>144</v>
       </c>
+      <c r="O35" s="27"/>
+      <c r="P35" s="27"/>
+      <c r="Q35" s="27"/>
       <c r="R35" s="20">
-        <f>IF(OR(M35="",N35=""),"",M35*N35)</f>
+        <f t="shared" si="2"/>
         <v>432</v>
       </c>
       <c r="S35" s="9" t="s">
@@ -3260,11 +3367,11 @@
       <c r="T35" s="9"/>
       <c r="U35" s="20"/>
       <c r="V35" s="20" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="W35" s="20" t="str">
-        <f>IF(OR(R35="",V35=""),"",R35-V35)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="X35" s="10" t="s">
@@ -3306,7 +3413,7 @@
       <c r="K36" s="13" t="s">
         <v>68</v>
       </c>
-      <c r="L36" s="26" t="s">
+      <c r="L36" s="24" t="s">
         <v>30</v>
       </c>
       <c r="M36" s="14">
@@ -3315,6 +3422,9 @@
       <c r="N36" s="21">
         <v>144</v>
       </c>
+      <c r="O36" s="27"/>
+      <c r="P36" s="27"/>
+      <c r="Q36" s="27"/>
       <c r="R36" s="21">
         <f>IF(OR(M36="",N36=""),"",M36*N36)</f>
         <v>576</v>
@@ -3325,11 +3435,11 @@
       <c r="T36" s="14"/>
       <c r="U36" s="21"/>
       <c r="V36" s="21" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="W36" s="21" t="str">
-        <f>IF(OR(R36="",V36=""),"",R36-V36)</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="X36" s="15" t="s">
@@ -3367,29 +3477,29 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:21" ht="21">
-      <c r="A1" s="24" t="s">
+      <c r="A1" s="25" t="s">
         <v>107</v>
       </c>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
-      <c r="D1" s="24"/>
-      <c r="E1" s="24"/>
-      <c r="F1" s="24"/>
-      <c r="G1" s="24"/>
-      <c r="H1" s="24"/>
-      <c r="I1" s="24"/>
-      <c r="J1" s="24"/>
-      <c r="K1" s="24"/>
-      <c r="L1" s="24"/>
-      <c r="M1" s="24"/>
-      <c r="N1" s="24"/>
-      <c r="O1" s="24"/>
-      <c r="P1" s="24"/>
-      <c r="Q1" s="24"/>
-      <c r="R1" s="24"/>
-      <c r="S1" s="24"/>
-      <c r="T1" s="24"/>
-      <c r="U1" s="24"/>
+      <c r="B1" s="25"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
+      <c r="E1" s="25"/>
+      <c r="F1" s="25"/>
+      <c r="G1" s="25"/>
+      <c r="H1" s="25"/>
+      <c r="I1" s="25"/>
+      <c r="J1" s="25"/>
+      <c r="K1" s="25"/>
+      <c r="L1" s="25"/>
+      <c r="M1" s="25"/>
+      <c r="N1" s="25"/>
+      <c r="O1" s="25"/>
+      <c r="P1" s="25"/>
+      <c r="Q1" s="25"/>
+      <c r="R1" s="25"/>
+      <c r="S1" s="25"/>
+      <c r="T1" s="25"/>
+      <c r="U1" s="25"/>
     </row>
     <row r="2" spans="1:21" ht="32">
       <c r="A2" s="3" t="s">
@@ -3645,7 +3755,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="6" spans="1:21" ht="28">
+    <row r="6" spans="1:21">
       <c r="A6" s="6" t="s">
         <v>22</v>
       </c>
@@ -4779,7 +4889,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="24" spans="1:21" ht="28">
+    <row r="24" spans="1:21">
       <c r="A24" s="6" t="s">
         <v>80</v>
       </c>
@@ -5472,7 +5582,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="35" spans="1:21" ht="28">
+    <row r="35" spans="1:21">
       <c r="A35" s="6" t="s">
         <v>80</v>
       </c>
@@ -5618,16 +5728,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="21">
-      <c r="A1" s="25" t="s">
+      <c r="A1" s="26" t="s">
         <v>149</v>
       </c>
-      <c r="B1" s="25"/>
-      <c r="C1" s="25"/>
-      <c r="D1" s="25"/>
-      <c r="E1" s="25"/>
-      <c r="F1" s="25"/>
-      <c r="G1" s="25"/>
-      <c r="H1" s="25"/>
+      <c r="B1" s="26"/>
+      <c r="C1" s="26"/>
+      <c r="D1" s="26"/>
+      <c r="E1" s="26"/>
+      <c r="F1" s="26"/>
+      <c r="G1" s="26"/>
+      <c r="H1" s="26"/>
     </row>
     <row r="2" spans="1:8" ht="32">
       <c r="A2" s="1" t="s">

</xml_diff>

<commit_message>
Added columns for existing luminaires (2)
</commit_message>
<xml_diff>
--- a/Building A B Lighting New.xlsx
+++ b/Building A B Lighting New.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10118"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pacopoon/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lsen906\Documents\Alpha_Design_17\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F31CB5C-A36D-7B42-966D-79C0DAF53044}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D764F81-86BA-4BC3-A730-A242110B5A33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="25840" windowHeight="15300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Building A" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="856" uniqueCount="186">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="891" uniqueCount="188">
   <si>
     <t>Building A — Lighting Place Schedule</t>
   </si>
@@ -593,13 +593,19 @@
   </si>
   <si>
     <t>Existing Luminaire (2)</t>
+  </si>
+  <si>
+    <t>Existing Qty (2)</t>
+  </si>
+  <si>
+    <t>Existing W each (2)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -618,6 +624,10 @@
     </font>
     <font>
       <sz val="10"/>
+      <name val="Carlito"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Carlito"/>
     </font>
   </fonts>
@@ -820,15 +830,15 @@
     <xf numFmtId="0" fontId="3" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1002,7 +1012,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:X36"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
+  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="2" width="10" customWidth="1"/>
     <col min="3" max="3" width="20" customWidth="1"/>
@@ -1021,32 +1031,32 @@
     <col min="21" max="21" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" ht="21">
-      <c r="A1" s="25" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="25"/>
-      <c r="C1" s="25"/>
-      <c r="D1" s="25"/>
-      <c r="E1" s="25"/>
-      <c r="F1" s="25"/>
-      <c r="G1" s="25"/>
-      <c r="H1" s="25"/>
-      <c r="I1" s="25"/>
-      <c r="J1" s="25"/>
-      <c r="K1" s="25"/>
-      <c r="L1" s="25"/>
-      <c r="M1" s="25"/>
-      <c r="N1" s="25"/>
-      <c r="O1" s="25"/>
-      <c r="P1" s="25"/>
-      <c r="Q1" s="25"/>
-      <c r="R1" s="25"/>
-      <c r="S1" s="25"/>
-      <c r="T1" s="25"/>
-      <c r="U1" s="25"/>
-    </row>
-    <row r="2" spans="1:24" ht="48">
+    <row r="1" spans="1:24" ht="20.25">
+      <c r="A1" s="27" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="27"/>
+      <c r="C1" s="27"/>
+      <c r="D1" s="27"/>
+      <c r="E1" s="27"/>
+      <c r="F1" s="27"/>
+      <c r="G1" s="27"/>
+      <c r="H1" s="27"/>
+      <c r="I1" s="27"/>
+      <c r="J1" s="27"/>
+      <c r="K1" s="27"/>
+      <c r="L1" s="27"/>
+      <c r="M1" s="27"/>
+      <c r="N1" s="27"/>
+      <c r="O1" s="27"/>
+      <c r="P1" s="27"/>
+      <c r="Q1" s="27"/>
+      <c r="R1" s="27"/>
+      <c r="S1" s="27"/>
+      <c r="T1" s="27"/>
+      <c r="U1" s="27"/>
+    </row>
+    <row r="2" spans="1:24" ht="45">
       <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
@@ -1120,7 +1130,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:24" ht="28">
+    <row r="3" spans="1:24" ht="25.5">
       <c r="A3" s="6" t="s">
         <v>22</v>
       </c>
@@ -1164,9 +1174,9 @@
       <c r="N3" s="20">
         <v>72</v>
       </c>
-      <c r="O3" s="27"/>
-      <c r="P3" s="27"/>
-      <c r="Q3" s="27"/>
+      <c r="O3" s="25"/>
+      <c r="P3" s="25"/>
+      <c r="Q3" s="25"/>
       <c r="R3" s="20">
         <f>IF(OR(M3="",N3=""),"",M3*N3)</f>
         <v>72</v>
@@ -1188,7 +1198,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="4" spans="1:24" ht="28">
+    <row r="4" spans="1:24" ht="25.5">
       <c r="A4" s="6" t="s">
         <v>22</v>
       </c>
@@ -1232,13 +1242,13 @@
       <c r="N4" s="20">
         <v>72</v>
       </c>
-      <c r="O4" s="28" t="s">
+      <c r="O4" s="26" t="s">
         <v>57</v>
       </c>
-      <c r="P4" s="27">
+      <c r="P4" s="25">
         <v>5</v>
       </c>
-      <c r="Q4" s="27">
+      <c r="Q4" s="25">
         <f>4*36</f>
         <v>144</v>
       </c>
@@ -1263,7 +1273,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="5" spans="1:24" ht="28">
+    <row r="5" spans="1:24" ht="25.5">
       <c r="A5" s="6" t="s">
         <v>22</v>
       </c>
@@ -1307,11 +1317,11 @@
       <c r="N5" s="20">
         <v>72</v>
       </c>
-      <c r="O5" s="28"/>
-      <c r="P5" s="27"/>
-      <c r="Q5" s="27"/>
+      <c r="O5" s="26"/>
+      <c r="P5" s="25"/>
+      <c r="Q5" s="25"/>
       <c r="R5" s="20">
-        <f t="shared" ref="R5:R36" si="2">IF(OR(M5="",N5=""),"",M5*N5)</f>
+        <f t="shared" ref="R5:R35" si="2">IF(OR(M5="",N5=""),"",M5*N5)</f>
         <v>72</v>
       </c>
       <c r="S5" s="9" t="s">
@@ -1331,7 +1341,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="6" spans="1:24" ht="28">
+    <row r="6" spans="1:24" ht="25.5">
       <c r="A6" s="6" t="s">
         <v>22</v>
       </c>
@@ -1375,9 +1385,9 @@
       <c r="N6" s="20">
         <v>72</v>
       </c>
-      <c r="O6" s="27"/>
-      <c r="P6" s="27"/>
-      <c r="Q6" s="27"/>
+      <c r="O6" s="25"/>
+      <c r="P6" s="25"/>
+      <c r="Q6" s="25"/>
       <c r="R6" s="20">
         <f t="shared" si="2"/>
         <v>72</v>
@@ -1399,7 +1409,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="7" spans="1:24" ht="28">
+    <row r="7" spans="1:24" ht="25.5">
       <c r="A7" s="6" t="s">
         <v>22</v>
       </c>
@@ -1443,9 +1453,9 @@
       <c r="N7" s="20">
         <v>72</v>
       </c>
-      <c r="O7" s="27"/>
-      <c r="P7" s="27"/>
-      <c r="Q7" s="27"/>
+      <c r="O7" s="25"/>
+      <c r="P7" s="25"/>
+      <c r="Q7" s="25"/>
       <c r="R7" s="20">
         <f t="shared" si="2"/>
         <v>72</v>
@@ -1467,7 +1477,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="8" spans="1:24" ht="28">
+    <row r="8" spans="1:24" ht="25.5">
       <c r="A8" s="6" t="s">
         <v>22</v>
       </c>
@@ -1511,9 +1521,9 @@
       <c r="N8" s="20">
         <v>144</v>
       </c>
-      <c r="O8" s="27"/>
-      <c r="P8" s="27"/>
-      <c r="Q8" s="27"/>
+      <c r="O8" s="25"/>
+      <c r="P8" s="25"/>
+      <c r="Q8" s="25"/>
       <c r="R8" s="20">
         <f t="shared" si="2"/>
         <v>288</v>
@@ -1535,7 +1545,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="9" spans="1:24" ht="28">
+    <row r="9" spans="1:24" ht="25.5">
       <c r="A9" s="6" t="s">
         <v>22</v>
       </c>
@@ -1579,9 +1589,9 @@
       <c r="N9" s="20">
         <v>144</v>
       </c>
-      <c r="O9" s="27"/>
-      <c r="P9" s="27"/>
-      <c r="Q9" s="27"/>
+      <c r="O9" s="25"/>
+      <c r="P9" s="25"/>
+      <c r="Q9" s="25"/>
       <c r="R9" s="20">
         <f t="shared" si="2"/>
         <v>288</v>
@@ -1603,7 +1613,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="10" spans="1:24" ht="28">
+    <row r="10" spans="1:24" ht="25.5">
       <c r="A10" s="6" t="s">
         <v>22</v>
       </c>
@@ -1647,13 +1657,13 @@
       <c r="N10" s="20">
         <v>72</v>
       </c>
-      <c r="O10" s="28" t="s">
+      <c r="O10" s="26" t="s">
         <v>57</v>
       </c>
-      <c r="P10" s="27">
+      <c r="P10" s="25">
         <v>4</v>
       </c>
-      <c r="Q10" s="27">
+      <c r="Q10" s="25">
         <f>4*36</f>
         <v>144</v>
       </c>
@@ -1678,7 +1688,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="11" spans="1:24" ht="28">
+    <row r="11" spans="1:24" ht="25.5">
       <c r="A11" s="6" t="s">
         <v>22</v>
       </c>
@@ -1722,9 +1732,9 @@
       <c r="N11" s="20">
         <v>144</v>
       </c>
-      <c r="O11" s="27"/>
-      <c r="P11" s="27"/>
-      <c r="Q11" s="27"/>
+      <c r="O11" s="25"/>
+      <c r="P11" s="25"/>
+      <c r="Q11" s="25"/>
       <c r="R11" s="20">
         <f t="shared" si="2"/>
         <v>288</v>
@@ -1746,7 +1756,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="12" spans="1:24" ht="28">
+    <row r="12" spans="1:24" ht="25.5">
       <c r="A12" s="6" t="s">
         <v>22</v>
       </c>
@@ -1790,9 +1800,9 @@
       <c r="N12" s="20">
         <v>144</v>
       </c>
-      <c r="O12" s="27"/>
-      <c r="P12" s="27"/>
-      <c r="Q12" s="27"/>
+      <c r="O12" s="25"/>
+      <c r="P12" s="25"/>
+      <c r="Q12" s="25"/>
       <c r="R12" s="20">
         <f t="shared" si="2"/>
         <v>576</v>
@@ -1814,7 +1824,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="13" spans="1:24" ht="28">
+    <row r="13" spans="1:24" ht="25.5">
       <c r="A13" s="6" t="s">
         <v>22</v>
       </c>
@@ -1858,9 +1868,9 @@
       <c r="N13" s="20">
         <v>144</v>
       </c>
-      <c r="O13" s="27"/>
-      <c r="P13" s="27"/>
-      <c r="Q13" s="27"/>
+      <c r="O13" s="25"/>
+      <c r="P13" s="25"/>
+      <c r="Q13" s="25"/>
       <c r="R13" s="20">
         <f t="shared" si="2"/>
         <v>576</v>
@@ -1882,7 +1892,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="14" spans="1:24" ht="28">
+    <row r="14" spans="1:24" ht="25.5">
       <c r="A14" s="6" t="s">
         <v>22</v>
       </c>
@@ -1926,9 +1936,9 @@
       <c r="N14" s="20">
         <v>144</v>
       </c>
-      <c r="O14" s="27"/>
-      <c r="P14" s="27"/>
-      <c r="Q14" s="27"/>
+      <c r="O14" s="25"/>
+      <c r="P14" s="25"/>
+      <c r="Q14" s="25"/>
       <c r="R14" s="20">
         <f t="shared" si="2"/>
         <v>864</v>
@@ -1950,7 +1960,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="15" spans="1:24" ht="28">
+    <row r="15" spans="1:24" ht="25.5">
       <c r="A15" s="6" t="s">
         <v>22</v>
       </c>
@@ -1994,9 +2004,9 @@
       <c r="N15" s="20">
         <v>144</v>
       </c>
-      <c r="O15" s="27"/>
-      <c r="P15" s="27"/>
-      <c r="Q15" s="27"/>
+      <c r="O15" s="25"/>
+      <c r="P15" s="25"/>
+      <c r="Q15" s="25"/>
       <c r="R15" s="20">
         <f t="shared" si="2"/>
         <v>432</v>
@@ -2018,7 +2028,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="16" spans="1:24" ht="28">
+    <row r="16" spans="1:24" ht="25.5">
       <c r="A16" s="6" t="s">
         <v>22</v>
       </c>
@@ -2062,9 +2072,9 @@
       <c r="N16" s="20">
         <v>144</v>
       </c>
-      <c r="O16" s="27"/>
-      <c r="P16" s="27"/>
-      <c r="Q16" s="27"/>
+      <c r="O16" s="25"/>
+      <c r="P16" s="25"/>
+      <c r="Q16" s="25"/>
       <c r="R16" s="20">
         <f t="shared" si="2"/>
         <v>432</v>
@@ -2086,7 +2096,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="17" spans="1:24" ht="28">
+    <row r="17" spans="1:24" ht="25.5">
       <c r="A17" s="6" t="s">
         <v>80</v>
       </c>
@@ -2130,9 +2140,9 @@
       <c r="N17" s="20">
         <v>72</v>
       </c>
-      <c r="O17" s="27"/>
-      <c r="P17" s="27"/>
-      <c r="Q17" s="27"/>
+      <c r="O17" s="25"/>
+      <c r="P17" s="25"/>
+      <c r="Q17" s="25"/>
       <c r="R17" s="20">
         <f t="shared" si="2"/>
         <v>72</v>
@@ -2154,7 +2164,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="18" spans="1:24" ht="28">
+    <row r="18" spans="1:24" ht="25.5">
       <c r="A18" s="6" t="s">
         <v>80</v>
       </c>
@@ -2198,9 +2208,9 @@
       <c r="N18" s="20">
         <v>72</v>
       </c>
-      <c r="O18" s="27"/>
-      <c r="P18" s="27"/>
-      <c r="Q18" s="27"/>
+      <c r="O18" s="25"/>
+      <c r="P18" s="25"/>
+      <c r="Q18" s="25"/>
       <c r="R18" s="20">
         <f t="shared" si="2"/>
         <v>288</v>
@@ -2222,7 +2232,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="19" spans="1:24" ht="28">
+    <row r="19" spans="1:24" ht="25.5">
       <c r="A19" s="6" t="s">
         <v>80</v>
       </c>
@@ -2266,9 +2276,9 @@
       <c r="N19" s="20">
         <v>144</v>
       </c>
-      <c r="O19" s="27"/>
-      <c r="P19" s="27"/>
-      <c r="Q19" s="27"/>
+      <c r="O19" s="25"/>
+      <c r="P19" s="25"/>
+      <c r="Q19" s="25"/>
       <c r="R19" s="20">
         <f t="shared" si="2"/>
         <v>288</v>
@@ -2290,7 +2300,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="20" spans="1:24" ht="28">
+    <row r="20" spans="1:24" ht="25.5">
       <c r="A20" s="6" t="s">
         <v>80</v>
       </c>
@@ -2334,9 +2344,9 @@
       <c r="N20" s="20">
         <v>144</v>
       </c>
-      <c r="O20" s="27"/>
-      <c r="P20" s="27"/>
-      <c r="Q20" s="27"/>
+      <c r="O20" s="25"/>
+      <c r="P20" s="25"/>
+      <c r="Q20" s="25"/>
       <c r="R20" s="20">
         <f t="shared" si="2"/>
         <v>1008</v>
@@ -2358,7 +2368,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="21" spans="1:24" ht="28">
+    <row r="21" spans="1:24" ht="25.5">
       <c r="A21" s="6" t="s">
         <v>80</v>
       </c>
@@ -2402,9 +2412,9 @@
       <c r="N21" s="20">
         <v>72</v>
       </c>
-      <c r="O21" s="27"/>
-      <c r="P21" s="27"/>
-      <c r="Q21" s="27"/>
+      <c r="O21" s="25"/>
+      <c r="P21" s="25"/>
+      <c r="Q21" s="25"/>
       <c r="R21" s="20">
         <f t="shared" si="2"/>
         <v>72</v>
@@ -2426,7 +2436,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="22" spans="1:24" ht="28">
+    <row r="22" spans="1:24" ht="25.5">
       <c r="A22" s="6" t="s">
         <v>80</v>
       </c>
@@ -2470,9 +2480,9 @@
       <c r="N22" s="20">
         <v>72</v>
       </c>
-      <c r="O22" s="27"/>
-      <c r="P22" s="27"/>
-      <c r="Q22" s="27"/>
+      <c r="O22" s="25"/>
+      <c r="P22" s="25"/>
+      <c r="Q22" s="25"/>
       <c r="R22" s="20">
         <f t="shared" si="2"/>
         <v>144</v>
@@ -2494,7 +2504,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="23" spans="1:24" ht="28">
+    <row r="23" spans="1:24" ht="25.5">
       <c r="A23" s="6" t="s">
         <v>80</v>
       </c>
@@ -2538,9 +2548,9 @@
       <c r="N23" s="20">
         <v>144</v>
       </c>
-      <c r="O23" s="27"/>
-      <c r="P23" s="27"/>
-      <c r="Q23" s="27"/>
+      <c r="O23" s="25"/>
+      <c r="P23" s="25"/>
+      <c r="Q23" s="25"/>
       <c r="R23" s="20">
         <f t="shared" si="2"/>
         <v>864</v>
@@ -2562,7 +2572,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="24" spans="1:24" ht="28">
+    <row r="24" spans="1:24" ht="25.5">
       <c r="A24" s="6" t="s">
         <v>80</v>
       </c>
@@ -2606,9 +2616,9 @@
       <c r="N24" s="20">
         <v>144</v>
       </c>
-      <c r="O24" s="27"/>
-      <c r="P24" s="27"/>
-      <c r="Q24" s="27"/>
+      <c r="O24" s="25"/>
+      <c r="P24" s="25"/>
+      <c r="Q24" s="25"/>
       <c r="R24" s="20">
         <f t="shared" si="2"/>
         <v>576</v>
@@ -2630,7 +2640,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="25" spans="1:24" ht="28">
+    <row r="25" spans="1:24" ht="25.5">
       <c r="A25" s="6" t="s">
         <v>80</v>
       </c>
@@ -2674,9 +2684,9 @@
       <c r="N25" s="20">
         <v>144</v>
       </c>
-      <c r="O25" s="27"/>
-      <c r="P25" s="27"/>
-      <c r="Q25" s="27"/>
+      <c r="O25" s="25"/>
+      <c r="P25" s="25"/>
+      <c r="Q25" s="25"/>
       <c r="R25" s="20">
         <f t="shared" si="2"/>
         <v>576</v>
@@ -2698,7 +2708,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="26" spans="1:24" ht="28">
+    <row r="26" spans="1:24" ht="25.5">
       <c r="A26" s="6" t="s">
         <v>80</v>
       </c>
@@ -2742,9 +2752,9 @@
       <c r="N26" s="20">
         <v>144</v>
       </c>
-      <c r="O26" s="27"/>
-      <c r="P26" s="27"/>
-      <c r="Q26" s="27"/>
+      <c r="O26" s="25"/>
+      <c r="P26" s="25"/>
+      <c r="Q26" s="25"/>
       <c r="R26" s="20">
         <f t="shared" si="2"/>
         <v>1152</v>
@@ -2766,7 +2776,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="27" spans="1:24" ht="28">
+    <row r="27" spans="1:24" ht="25.5">
       <c r="A27" s="6" t="s">
         <v>80</v>
       </c>
@@ -2810,9 +2820,9 @@
       <c r="N27" s="20">
         <v>72</v>
       </c>
-      <c r="O27" s="27"/>
-      <c r="P27" s="27"/>
-      <c r="Q27" s="27"/>
+      <c r="O27" s="25"/>
+      <c r="P27" s="25"/>
+      <c r="Q27" s="25"/>
       <c r="R27" s="20">
         <f t="shared" si="2"/>
         <v>576</v>
@@ -2834,7 +2844,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="28" spans="1:24" ht="28">
+    <row r="28" spans="1:24" ht="25.5">
       <c r="A28" s="6" t="s">
         <v>80</v>
       </c>
@@ -2878,9 +2888,9 @@
       <c r="N28" s="20">
         <v>144</v>
       </c>
-      <c r="O28" s="27"/>
-      <c r="P28" s="27"/>
-      <c r="Q28" s="27"/>
+      <c r="O28" s="25"/>
+      <c r="P28" s="25"/>
+      <c r="Q28" s="25"/>
       <c r="R28" s="20">
         <f t="shared" si="2"/>
         <v>1152</v>
@@ -2902,7 +2912,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="29" spans="1:24" ht="28">
+    <row r="29" spans="1:24" ht="25.5">
       <c r="A29" s="6" t="s">
         <v>80</v>
       </c>
@@ -2946,9 +2956,9 @@
       <c r="N29" s="20">
         <v>72</v>
       </c>
-      <c r="O29" s="27"/>
-      <c r="P29" s="27"/>
-      <c r="Q29" s="27"/>
+      <c r="O29" s="25"/>
+      <c r="P29" s="25"/>
+      <c r="Q29" s="25"/>
       <c r="R29" s="20">
         <f t="shared" si="2"/>
         <v>72</v>
@@ -2970,7 +2980,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="30" spans="1:24" ht="28">
+    <row r="30" spans="1:24" ht="25.5">
       <c r="A30" s="6" t="s">
         <v>80</v>
       </c>
@@ -3014,9 +3024,9 @@
       <c r="N30" s="20">
         <v>144</v>
       </c>
-      <c r="O30" s="27"/>
-      <c r="P30" s="27"/>
-      <c r="Q30" s="27"/>
+      <c r="O30" s="25"/>
+      <c r="P30" s="25"/>
+      <c r="Q30" s="25"/>
       <c r="R30" s="20">
         <f t="shared" si="2"/>
         <v>576</v>
@@ -3038,7 +3048,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="31" spans="1:24" ht="28">
+    <row r="31" spans="1:24" ht="25.5">
       <c r="A31" s="6" t="s">
         <v>80</v>
       </c>
@@ -3082,9 +3092,9 @@
       <c r="N31" s="20">
         <v>144</v>
       </c>
-      <c r="O31" s="27"/>
-      <c r="P31" s="27"/>
-      <c r="Q31" s="27"/>
+      <c r="O31" s="25"/>
+      <c r="P31" s="25"/>
+      <c r="Q31" s="25"/>
       <c r="R31" s="20">
         <f t="shared" si="2"/>
         <v>576</v>
@@ -3106,7 +3116,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="32" spans="1:24" ht="28">
+    <row r="32" spans="1:24" ht="25.5">
       <c r="A32" s="6" t="s">
         <v>80</v>
       </c>
@@ -3150,9 +3160,9 @@
       <c r="N32" s="20">
         <v>144</v>
       </c>
-      <c r="O32" s="27"/>
-      <c r="P32" s="27"/>
-      <c r="Q32" s="27"/>
+      <c r="O32" s="25"/>
+      <c r="P32" s="25"/>
+      <c r="Q32" s="25"/>
       <c r="R32" s="20">
         <f t="shared" si="2"/>
         <v>576</v>
@@ -3174,7 +3184,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="33" spans="1:24" ht="28">
+    <row r="33" spans="1:24" ht="25.5">
       <c r="A33" s="6" t="s">
         <v>80</v>
       </c>
@@ -3218,9 +3228,9 @@
       <c r="N33" s="20">
         <v>72</v>
       </c>
-      <c r="O33" s="27"/>
-      <c r="P33" s="27"/>
-      <c r="Q33" s="27"/>
+      <c r="O33" s="25"/>
+      <c r="P33" s="25"/>
+      <c r="Q33" s="25"/>
       <c r="R33" s="20">
         <f t="shared" si="2"/>
         <v>72</v>
@@ -3242,7 +3252,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="34" spans="1:24" ht="28">
+    <row r="34" spans="1:24" ht="25.5">
       <c r="A34" s="6" t="s">
         <v>80</v>
       </c>
@@ -3286,9 +3296,9 @@
       <c r="N34" s="20">
         <v>72</v>
       </c>
-      <c r="O34" s="27"/>
-      <c r="P34" s="27"/>
-      <c r="Q34" s="27"/>
+      <c r="O34" s="25"/>
+      <c r="P34" s="25"/>
+      <c r="Q34" s="25"/>
       <c r="R34" s="20">
         <f t="shared" si="2"/>
         <v>72</v>
@@ -3310,7 +3320,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="35" spans="1:24" ht="28">
+    <row r="35" spans="1:24" ht="25.5">
       <c r="A35" s="6" t="s">
         <v>80</v>
       </c>
@@ -3354,9 +3364,9 @@
       <c r="N35" s="20">
         <v>144</v>
       </c>
-      <c r="O35" s="27"/>
-      <c r="P35" s="27"/>
-      <c r="Q35" s="27"/>
+      <c r="O35" s="25"/>
+      <c r="P35" s="25"/>
+      <c r="Q35" s="25"/>
       <c r="R35" s="20">
         <f t="shared" si="2"/>
         <v>432</v>
@@ -3378,7 +3388,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="36" spans="1:24" ht="28">
+    <row r="36" spans="1:24" ht="25.5">
       <c r="A36" s="11" t="s">
         <v>80</v>
       </c>
@@ -3422,9 +3432,9 @@
       <c r="N36" s="21">
         <v>144</v>
       </c>
-      <c r="O36" s="27"/>
-      <c r="P36" s="27"/>
-      <c r="Q36" s="27"/>
+      <c r="O36" s="25"/>
+      <c r="P36" s="25"/>
+      <c r="Q36" s="25"/>
       <c r="R36" s="21">
         <f>IF(OR(M36="",N36=""),"",M36*N36)</f>
         <v>576</v>
@@ -3456,8 +3466,8 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:U36"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
+  <dimension ref="A1:X37"/>
+  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="2" width="10" customWidth="1"/>
     <col min="3" max="3" width="20" customWidth="1"/>
@@ -3470,38 +3480,44 @@
     <col min="12" max="12" width="22" customWidth="1"/>
     <col min="13" max="14" width="12" customWidth="1"/>
     <col min="15" max="15" width="14" customWidth="1"/>
-    <col min="16" max="16" width="24" customWidth="1"/>
-    <col min="17" max="18" width="12" customWidth="1"/>
-    <col min="19" max="20" width="14" customWidth="1"/>
-    <col min="21" max="21" width="16" customWidth="1"/>
+    <col min="16" max="16" width="15.625" customWidth="1"/>
+    <col min="17" max="17" width="12" customWidth="1"/>
+    <col min="18" max="18" width="14" customWidth="1"/>
+    <col min="19" max="19" width="24" customWidth="1"/>
+    <col min="20" max="21" width="12" customWidth="1"/>
+    <col min="22" max="23" width="14" customWidth="1"/>
+    <col min="24" max="24" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" ht="21">
-      <c r="A1" s="25" t="s">
+    <row r="1" spans="1:24" ht="20.25">
+      <c r="A1" s="27" t="s">
         <v>107</v>
       </c>
-      <c r="B1" s="25"/>
-      <c r="C1" s="25"/>
-      <c r="D1" s="25"/>
-      <c r="E1" s="25"/>
-      <c r="F1" s="25"/>
-      <c r="G1" s="25"/>
-      <c r="H1" s="25"/>
-      <c r="I1" s="25"/>
-      <c r="J1" s="25"/>
-      <c r="K1" s="25"/>
-      <c r="L1" s="25"/>
-      <c r="M1" s="25"/>
-      <c r="N1" s="25"/>
-      <c r="O1" s="25"/>
-      <c r="P1" s="25"/>
-      <c r="Q1" s="25"/>
-      <c r="R1" s="25"/>
-      <c r="S1" s="25"/>
-      <c r="T1" s="25"/>
-      <c r="U1" s="25"/>
-    </row>
-    <row r="2" spans="1:21" ht="32">
+      <c r="B1" s="27"/>
+      <c r="C1" s="27"/>
+      <c r="D1" s="27"/>
+      <c r="E1" s="27"/>
+      <c r="F1" s="27"/>
+      <c r="G1" s="27"/>
+      <c r="H1" s="27"/>
+      <c r="I1" s="27"/>
+      <c r="J1" s="27"/>
+      <c r="K1" s="27"/>
+      <c r="L1" s="27"/>
+      <c r="M1" s="27"/>
+      <c r="N1" s="27"/>
+      <c r="O1" s="27"/>
+      <c r="P1" s="27"/>
+      <c r="Q1" s="27"/>
+      <c r="R1" s="27"/>
+      <c r="S1" s="27"/>
+      <c r="T1" s="27"/>
+      <c r="U1" s="27"/>
+      <c r="V1" s="27"/>
+      <c r="W1" s="27"/>
+      <c r="X1" s="27"/>
+    </row>
+    <row r="2" spans="1:24" ht="30">
       <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
@@ -3545,28 +3561,37 @@
         <v>14</v>
       </c>
       <c r="O2" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="P2" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="Q2" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="R2" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="P2" s="4" t="s">
+      <c r="S2" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="Q2" s="4" t="s">
+      <c r="T2" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="R2" s="4" t="s">
+      <c r="U2" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="S2" s="4" t="s">
+      <c r="V2" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="T2" s="4" t="s">
+      <c r="W2" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="U2" s="5" t="s">
+      <c r="X2" s="5" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:21">
+    <row r="3" spans="1:24">
       <c r="A3" s="6" t="s">
         <v>22</v>
       </c>
@@ -3586,7 +3611,7 @@
         <v>80</v>
       </c>
       <c r="G3" s="18">
-        <f t="shared" ref="G3:G36" si="0">ROUND(F3/0.8,0)</f>
+        <f t="shared" ref="G3:G37" si="0">ROUND(F3/0.8,0)</f>
         <v>100</v>
       </c>
       <c r="H3" s="8" t="s">
@@ -3604,32 +3629,45 @@
       <c r="L3" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="M3" s="9"/>
+      <c r="M3" s="9">
+        <v>1</v>
+      </c>
       <c r="N3" s="20">
+        <f>2*36*M3</f>
         <v>72</v>
       </c>
-      <c r="O3" s="20" t="str">
-        <f t="shared" ref="O3:O36" si="1">IF(OR(M3="",N3=""),"",M3*N3)</f>
-        <v/>
-      </c>
-      <c r="P3" s="9" t="s">
+      <c r="O3" s="26" t="s">
+        <v>57</v>
+      </c>
+      <c r="P3" s="25">
+        <v>0</v>
+      </c>
+      <c r="Q3" s="25">
+        <f>4*36*P3</f>
+        <v>0</v>
+      </c>
+      <c r="R3" s="20">
+        <f>N3+Q3</f>
+        <v>72</v>
+      </c>
+      <c r="S3" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="Q3" s="9"/>
-      <c r="R3" s="20"/>
-      <c r="S3" s="20" t="str">
-        <f t="shared" ref="S3:S36" si="2">IF(OR(Q3="",R3=""),"",Q3*R3)</f>
-        <v/>
-      </c>
-      <c r="T3" s="20" t="str">
-        <f t="shared" ref="T3:T36" si="3">IF(OR(O3="",S3=""),"",O3-S3)</f>
-        <v/>
-      </c>
-      <c r="U3" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="4" spans="1:21">
+      <c r="T3" s="9"/>
+      <c r="U3" s="20"/>
+      <c r="V3" s="20" t="str">
+        <f t="shared" ref="V3:V37" si="1">IF(OR(T3="",U3=""),"",T3*U3)</f>
+        <v/>
+      </c>
+      <c r="W3" s="20" t="str">
+        <f t="shared" ref="W3:W37" si="2">IF(OR(R3="",V3=""),"",R3-V3)</f>
+        <v/>
+      </c>
+      <c r="X3" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="4" spans="1:24">
       <c r="A4" s="6" t="s">
         <v>22</v>
       </c>
@@ -3667,32 +3705,45 @@
       <c r="L4" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="M4" s="9"/>
+      <c r="M4" s="9">
+        <v>2</v>
+      </c>
       <c r="N4" s="20">
-        <v>72</v>
-      </c>
-      <c r="O4" s="20" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="P4" s="9" t="s">
+        <f t="shared" ref="N4:N23" si="3">2*36*M4</f>
+        <v>144</v>
+      </c>
+      <c r="O4" s="26" t="s">
+        <v>57</v>
+      </c>
+      <c r="P4" s="25">
+        <v>5</v>
+      </c>
+      <c r="Q4" s="25">
+        <f t="shared" ref="Q4:Q23" si="4">4*36*P4</f>
+        <v>720</v>
+      </c>
+      <c r="R4" s="20">
+        <f t="shared" ref="R4:R23" si="5">N4+Q4</f>
+        <v>864</v>
+      </c>
+      <c r="S4" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="Q4" s="9"/>
-      <c r="R4" s="20"/>
-      <c r="S4" s="20" t="str">
+      <c r="T4" s="9"/>
+      <c r="U4" s="20"/>
+      <c r="V4" s="20" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="W4" s="20" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="T4" s="20" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="U4" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="5" spans="1:21" ht="28">
+      <c r="X4" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="5" spans="1:24" ht="25.5">
       <c r="A5" s="6" t="s">
         <v>22</v>
       </c>
@@ -3730,32 +3781,45 @@
       <c r="L5" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="M5" s="9"/>
+      <c r="M5" s="9">
+        <v>0</v>
+      </c>
       <c r="N5" s="20">
-        <v>72</v>
-      </c>
-      <c r="O5" s="20" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="P5" s="9" t="s">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="O5" s="26" t="s">
+        <v>57</v>
+      </c>
+      <c r="P5" s="25">
+        <v>1</v>
+      </c>
+      <c r="Q5" s="25">
+        <f t="shared" si="4"/>
+        <v>144</v>
+      </c>
+      <c r="R5" s="20">
+        <f t="shared" si="5"/>
+        <v>144</v>
+      </c>
+      <c r="S5" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="Q5" s="9"/>
-      <c r="R5" s="20"/>
-      <c r="S5" s="20" t="str">
+      <c r="T5" s="9"/>
+      <c r="U5" s="20"/>
+      <c r="V5" s="20" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="W5" s="20" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="T5" s="20" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="U5" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="6" spans="1:21">
+      <c r="X5" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="6" spans="1:24" ht="25.5">
       <c r="A6" s="6" t="s">
         <v>22</v>
       </c>
@@ -3793,32 +3857,45 @@
       <c r="L6" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="M6" s="9"/>
+      <c r="M6" s="9">
+        <v>1</v>
+      </c>
       <c r="N6" s="20">
+        <f t="shared" si="3"/>
         <v>72</v>
       </c>
-      <c r="O6" s="20" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="P6" s="9" t="s">
+      <c r="O6" s="26" t="s">
+        <v>57</v>
+      </c>
+      <c r="P6" s="25">
+        <v>0</v>
+      </c>
+      <c r="Q6" s="25">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="R6" s="20">
+        <f t="shared" si="5"/>
+        <v>72</v>
+      </c>
+      <c r="S6" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="Q6" s="9"/>
-      <c r="R6" s="20"/>
-      <c r="S6" s="20" t="str">
+      <c r="T6" s="9"/>
+      <c r="U6" s="20"/>
+      <c r="V6" s="20" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="W6" s="20" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="T6" s="20" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="U6" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="7" spans="1:21" ht="28">
+      <c r="X6" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="7" spans="1:24" ht="25.5">
       <c r="A7" s="6" t="s">
         <v>22</v>
       </c>
@@ -3856,32 +3933,45 @@
       <c r="L7" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="M7" s="9"/>
+      <c r="M7" s="9">
+        <v>1</v>
+      </c>
       <c r="N7" s="20">
+        <f t="shared" si="3"/>
         <v>72</v>
       </c>
-      <c r="O7" s="20" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="P7" s="9" t="s">
+      <c r="O7" s="26" t="s">
+        <v>57</v>
+      </c>
+      <c r="P7" s="25">
+        <v>0</v>
+      </c>
+      <c r="Q7" s="25">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="R7" s="20">
+        <f t="shared" si="5"/>
+        <v>72</v>
+      </c>
+      <c r="S7" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="Q7" s="9"/>
-      <c r="R7" s="20"/>
-      <c r="S7" s="20" t="str">
+      <c r="T7" s="9"/>
+      <c r="U7" s="20"/>
+      <c r="V7" s="20" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="W7" s="20" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="T7" s="20" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="U7" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="8" spans="1:21" ht="28">
+      <c r="X7" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="8" spans="1:24" ht="25.5">
       <c r="A8" s="6" t="s">
         <v>22</v>
       </c>
@@ -3919,32 +4009,45 @@
       <c r="L8" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="M8" s="9"/>
+      <c r="M8" s="9">
+        <v>1</v>
+      </c>
       <c r="N8" s="20">
+        <f t="shared" si="3"/>
         <v>72</v>
       </c>
-      <c r="O8" s="20" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="P8" s="9" t="s">
+      <c r="O8" s="26" t="s">
+        <v>57</v>
+      </c>
+      <c r="P8" s="25">
+        <v>0</v>
+      </c>
+      <c r="Q8" s="25">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="R8" s="20">
+        <f t="shared" si="5"/>
+        <v>72</v>
+      </c>
+      <c r="S8" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="Q8" s="9"/>
-      <c r="R8" s="20"/>
-      <c r="S8" s="20" t="str">
+      <c r="T8" s="9"/>
+      <c r="U8" s="20"/>
+      <c r="V8" s="20" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="W8" s="20" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="T8" s="20" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="U8" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="9" spans="1:21" ht="28">
+      <c r="X8" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="9" spans="1:24" ht="25.5">
       <c r="A9" s="6" t="s">
         <v>22</v>
       </c>
@@ -3982,32 +4085,45 @@
       <c r="L9" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="M9" s="9"/>
+      <c r="M9" s="9">
+        <v>1</v>
+      </c>
       <c r="N9" s="20">
+        <f t="shared" si="3"/>
         <v>72</v>
       </c>
-      <c r="O9" s="20" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="P9" s="9" t="s">
+      <c r="O9" s="26" t="s">
+        <v>57</v>
+      </c>
+      <c r="P9" s="25">
+        <v>0</v>
+      </c>
+      <c r="Q9" s="25">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="R9" s="20">
+        <f t="shared" si="5"/>
+        <v>72</v>
+      </c>
+      <c r="S9" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="Q9" s="9"/>
-      <c r="R9" s="20"/>
-      <c r="S9" s="20" t="str">
+      <c r="T9" s="9"/>
+      <c r="U9" s="20"/>
+      <c r="V9" s="20" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="W9" s="20" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="T9" s="20" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="U9" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="10" spans="1:21">
+      <c r="X9" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="10" spans="1:24">
       <c r="A10" s="6" t="s">
         <v>22</v>
       </c>
@@ -4043,39 +4159,52 @@
         <v>68</v>
       </c>
       <c r="L10" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="M10" s="9">
+        <v>0</v>
+      </c>
+      <c r="N10" s="20">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="O10" s="26" t="s">
         <v>57</v>
       </c>
-      <c r="M10" s="9"/>
-      <c r="N10" s="20">
-        <v>144</v>
-      </c>
-      <c r="O10" s="20" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="P10" s="9" t="s">
+      <c r="P10" s="25">
+        <v>4</v>
+      </c>
+      <c r="Q10" s="25">
+        <f t="shared" si="4"/>
+        <v>576</v>
+      </c>
+      <c r="R10" s="20">
+        <f t="shared" si="5"/>
+        <v>576</v>
+      </c>
+      <c r="S10" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="Q10" s="9"/>
-      <c r="R10" s="20"/>
-      <c r="S10" s="20" t="str">
+      <c r="T10" s="9"/>
+      <c r="U10" s="20"/>
+      <c r="V10" s="20" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="W10" s="20" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="T10" s="20" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="U10" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="11" spans="1:21">
+      <c r="X10" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="11" spans="1:24">
       <c r="A11" s="6" t="s">
         <v>22</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="C11" s="7" t="s">
         <v>70</v>
@@ -4090,7 +4219,7 @@
         <v>320</v>
       </c>
       <c r="G11" s="18">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="G11" si="6">ROUND(F11/0.8,0)</f>
         <v>400</v>
       </c>
       <c r="H11" s="8" t="s">
@@ -4106,45 +4235,58 @@
         <v>68</v>
       </c>
       <c r="L11" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="M11" s="9">
+        <v>0</v>
+      </c>
+      <c r="N11" s="20">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="O11" s="26" t="s">
         <v>57</v>
       </c>
-      <c r="M11" s="9"/>
-      <c r="N11" s="20">
-        <v>144</v>
-      </c>
-      <c r="O11" s="20" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="P11" s="9" t="s">
+      <c r="P11" s="25">
+        <v>2</v>
+      </c>
+      <c r="Q11" s="25">
+        <f t="shared" si="4"/>
+        <v>288</v>
+      </c>
+      <c r="R11" s="20">
+        <f>N11+Q11</f>
+        <v>288</v>
+      </c>
+      <c r="S11" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="Q11" s="9"/>
-      <c r="R11" s="20"/>
-      <c r="S11" s="20" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="T11" s="20" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="U11" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="12" spans="1:21">
+      <c r="T11" s="9"/>
+      <c r="U11" s="20"/>
+      <c r="V11" s="20" t="str">
+        <f t="shared" ref="V11" si="7">IF(OR(T11="",U11=""),"",T11*U11)</f>
+        <v/>
+      </c>
+      <c r="W11" s="20" t="str">
+        <f t="shared" ref="W11" si="8">IF(OR(R11="",V11=""),"",R11-V11)</f>
+        <v/>
+      </c>
+      <c r="X11" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="12" spans="1:24">
       <c r="A12" s="6" t="s">
         <v>22</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>85</v>
+        <v>70</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>86</v>
+        <v>71</v>
       </c>
       <c r="E12" s="16">
         <v>0.7</v>
@@ -4169,45 +4311,58 @@
         <v>68</v>
       </c>
       <c r="L12" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="M12" s="9">
+        <v>0</v>
+      </c>
+      <c r="N12" s="20">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="O12" s="26" t="s">
         <v>57</v>
       </c>
-      <c r="M12" s="9"/>
-      <c r="N12" s="20">
-        <v>144</v>
-      </c>
-      <c r="O12" s="20" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="P12" s="9" t="s">
+      <c r="P12" s="25">
+        <v>6</v>
+      </c>
+      <c r="Q12" s="25">
+        <f t="shared" si="4"/>
+        <v>864</v>
+      </c>
+      <c r="R12" s="20">
+        <f t="shared" si="5"/>
+        <v>864</v>
+      </c>
+      <c r="S12" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="Q12" s="9"/>
-      <c r="R12" s="20"/>
-      <c r="S12" s="20" t="str">
+      <c r="T12" s="9"/>
+      <c r="U12" s="20"/>
+      <c r="V12" s="20" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="W12" s="20" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="T12" s="20" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="U12" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="13" spans="1:21">
+      <c r="X12" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="13" spans="1:24">
       <c r="A13" s="6" t="s">
         <v>22</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>51</v>
+        <v>85</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>52</v>
+        <v>86</v>
       </c>
       <c r="E13" s="16">
         <v>0.7</v>
@@ -4223,117 +4378,143 @@
         <v>53</v>
       </c>
       <c r="I13" s="8" t="s">
-        <v>54</v>
+        <v>66</v>
       </c>
       <c r="J13" s="8" t="s">
-        <v>55</v>
+        <v>67</v>
       </c>
       <c r="K13" s="8" t="s">
-        <v>56</v>
+        <v>68</v>
       </c>
       <c r="L13" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="M13" s="9">
+        <v>0</v>
+      </c>
+      <c r="N13" s="20">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="O13" s="26" t="s">
         <v>57</v>
       </c>
-      <c r="M13" s="9"/>
-      <c r="N13" s="20">
-        <v>144</v>
-      </c>
-      <c r="O13" s="20" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="P13" s="9" t="s">
+      <c r="P13" s="25">
+        <v>2</v>
+      </c>
+      <c r="Q13" s="25">
+        <f t="shared" si="4"/>
+        <v>288</v>
+      </c>
+      <c r="R13" s="20">
+        <f t="shared" si="5"/>
+        <v>288</v>
+      </c>
+      <c r="S13" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="Q13" s="9"/>
-      <c r="R13" s="20"/>
-      <c r="S13" s="20" t="str">
+      <c r="T13" s="9"/>
+      <c r="U13" s="20"/>
+      <c r="V13" s="20" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="W13" s="20" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="T13" s="20" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="U13" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="14" spans="1:21">
+      <c r="X13" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="14" spans="1:24" ht="25.5">
       <c r="A14" s="6" t="s">
         <v>22</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>120</v>
+        <v>51</v>
       </c>
       <c r="D14" s="7" t="s">
-        <v>121</v>
+        <v>52</v>
       </c>
       <c r="E14" s="16">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="F14" s="18">
-        <v>40</v>
+        <v>320</v>
       </c>
       <c r="G14" s="18">
         <f t="shared" si="0"/>
-        <v>50</v>
+        <v>400</v>
       </c>
       <c r="H14" s="8" t="s">
-        <v>26</v>
+        <v>53</v>
       </c>
       <c r="I14" s="8" t="s">
-        <v>36</v>
+        <v>54</v>
       </c>
       <c r="J14" s="8" t="s">
-        <v>37</v>
+        <v>55</v>
       </c>
       <c r="K14" s="8" t="s">
-        <v>38</v>
+        <v>56</v>
       </c>
       <c r="L14" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="M14" s="9"/>
+      <c r="M14" s="9">
+        <v>0</v>
+      </c>
       <c r="N14" s="20">
-        <v>72</v>
-      </c>
-      <c r="O14" s="20" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="P14" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="Q14" s="9"/>
-      <c r="R14" s="20"/>
-      <c r="S14" s="20" t="str">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="O14" s="26" t="s">
+        <v>57</v>
+      </c>
+      <c r="P14" s="25">
+        <v>3</v>
+      </c>
+      <c r="Q14" s="25">
+        <f t="shared" si="4"/>
+        <v>432</v>
+      </c>
+      <c r="R14" s="20">
+        <f t="shared" si="5"/>
+        <v>432</v>
+      </c>
+      <c r="S14" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="T14" s="9"/>
+      <c r="U14" s="20"/>
+      <c r="V14" s="20" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="W14" s="20" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="T14" s="20" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="U14" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="15" spans="1:21" ht="28">
+      <c r="X14" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="15" spans="1:24">
       <c r="A15" s="6" t="s">
         <v>22</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>108</v>
+        <v>120</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>109</v>
+        <v>121</v>
       </c>
       <c r="E15" s="16">
         <v>0</v>
@@ -4346,120 +4527,146 @@
         <v>50</v>
       </c>
       <c r="H15" s="8" t="s">
-        <v>42</v>
+        <v>26</v>
       </c>
       <c r="I15" s="8" t="s">
-        <v>110</v>
+        <v>36</v>
       </c>
       <c r="J15" s="8" t="s">
-        <v>111</v>
+        <v>37</v>
       </c>
       <c r="K15" s="8" t="s">
-        <v>112</v>
+        <v>38</v>
       </c>
       <c r="L15" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="M15" s="9"/>
+      <c r="M15" s="9">
+        <v>0</v>
+      </c>
       <c r="N15" s="20">
-        <v>72</v>
-      </c>
-      <c r="O15" s="20" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="P15" s="9" t="s">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="O15" s="26" t="s">
+        <v>57</v>
+      </c>
+      <c r="P15" s="25">
+        <v>2</v>
+      </c>
+      <c r="Q15" s="25">
+        <f t="shared" si="4"/>
+        <v>288</v>
+      </c>
+      <c r="R15" s="20">
+        <f t="shared" si="5"/>
+        <v>288</v>
+      </c>
+      <c r="S15" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="Q15" s="9"/>
-      <c r="R15" s="20"/>
-      <c r="S15" s="20" t="str">
+      <c r="T15" s="9"/>
+      <c r="U15" s="20"/>
+      <c r="V15" s="20" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="W15" s="20" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="T15" s="20" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="U15" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="16" spans="1:21" ht="28">
+      <c r="X15" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="16" spans="1:24" ht="25.5">
       <c r="A16" s="6" t="s">
         <v>22</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>122</v>
+        <v>77</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>123</v>
+        <v>108</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>124</v>
+        <v>109</v>
       </c>
       <c r="E16" s="16">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="F16" s="18">
-        <v>320</v>
+        <v>40</v>
       </c>
       <c r="G16" s="18">
         <f t="shared" si="0"/>
-        <v>400</v>
+        <v>50</v>
       </c>
       <c r="H16" s="8" t="s">
-        <v>53</v>
+        <v>42</v>
       </c>
       <c r="I16" s="8" t="s">
-        <v>125</v>
+        <v>110</v>
       </c>
       <c r="J16" s="8" t="s">
-        <v>126</v>
+        <v>111</v>
       </c>
       <c r="K16" s="8" t="s">
-        <v>127</v>
+        <v>112</v>
       </c>
       <c r="L16" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="M16" s="9">
+        <v>0</v>
+      </c>
+      <c r="N16" s="20">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="O16" s="26" t="s">
         <v>57</v>
       </c>
-      <c r="M16" s="9"/>
-      <c r="N16" s="20">
+      <c r="P16" s="25">
+        <v>1</v>
+      </c>
+      <c r="Q16" s="25">
+        <f t="shared" si="4"/>
         <v>144</v>
       </c>
-      <c r="O16" s="20" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="P16" s="9" t="s">
-        <v>58</v>
-      </c>
-      <c r="Q16" s="9"/>
-      <c r="R16" s="20"/>
-      <c r="S16" s="20" t="str">
+      <c r="R16" s="20">
+        <f t="shared" si="5"/>
+        <v>144</v>
+      </c>
+      <c r="S16" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="T16" s="9"/>
+      <c r="U16" s="20"/>
+      <c r="V16" s="20" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="W16" s="20" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="T16" s="20" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="U16" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="17" spans="1:21">
+      <c r="X16" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="17" spans="1:24" ht="25.5">
       <c r="A17" s="6" t="s">
         <v>22</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>51</v>
+        <v>123</v>
       </c>
       <c r="D17" s="7" t="s">
-        <v>52</v>
+        <v>124</v>
       </c>
       <c r="E17" s="16">
         <v>0.7</v>
@@ -4475,180 +4682,219 @@
         <v>53</v>
       </c>
       <c r="I17" s="8" t="s">
-        <v>54</v>
+        <v>125</v>
       </c>
       <c r="J17" s="8" t="s">
-        <v>55</v>
+        <v>126</v>
       </c>
       <c r="K17" s="8" t="s">
-        <v>56</v>
+        <v>127</v>
       </c>
       <c r="L17" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="M17" s="9">
+        <v>0</v>
+      </c>
+      <c r="N17" s="20">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="O17" s="26" t="s">
         <v>57</v>
       </c>
-      <c r="M17" s="9"/>
-      <c r="N17" s="20">
-        <v>144</v>
-      </c>
-      <c r="O17" s="20" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="P17" s="9" t="s">
+      <c r="P17" s="25">
+        <v>4</v>
+      </c>
+      <c r="Q17" s="25">
+        <f t="shared" si="4"/>
+        <v>576</v>
+      </c>
+      <c r="R17" s="20">
+        <f t="shared" si="5"/>
+        <v>576</v>
+      </c>
+      <c r="S17" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="Q17" s="9"/>
-      <c r="R17" s="20"/>
-      <c r="S17" s="20" t="str">
+      <c r="T17" s="9"/>
+      <c r="U17" s="20"/>
+      <c r="V17" s="20" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="W17" s="20" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="T17" s="20" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="U17" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="18" spans="1:21">
+      <c r="X17" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="18" spans="1:24" ht="25.5">
       <c r="A18" s="6" t="s">
         <v>22</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="D18" s="7" t="s">
-        <v>62</v>
+        <v>52</v>
       </c>
       <c r="E18" s="16">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="F18" s="18">
-        <v>40</v>
+        <v>320</v>
       </c>
       <c r="G18" s="18">
         <f t="shared" si="0"/>
-        <v>50</v>
+        <v>400</v>
       </c>
       <c r="H18" s="8" t="s">
-        <v>26</v>
+        <v>53</v>
       </c>
       <c r="I18" s="8" t="s">
-        <v>36</v>
+        <v>54</v>
       </c>
       <c r="J18" s="8" t="s">
-        <v>37</v>
+        <v>55</v>
       </c>
       <c r="K18" s="8" t="s">
-        <v>38</v>
+        <v>56</v>
       </c>
       <c r="L18" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="M18" s="9"/>
+      <c r="M18" s="9">
+        <v>0</v>
+      </c>
       <c r="N18" s="20">
-        <v>72</v>
-      </c>
-      <c r="O18" s="20" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="P18" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="Q18" s="9"/>
-      <c r="R18" s="20"/>
-      <c r="S18" s="20" t="str">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="O18" s="26" t="s">
+        <v>57</v>
+      </c>
+      <c r="P18" s="25">
+        <v>2</v>
+      </c>
+      <c r="Q18" s="25">
+        <f t="shared" si="4"/>
+        <v>288</v>
+      </c>
+      <c r="R18" s="20">
+        <f t="shared" si="5"/>
+        <v>288</v>
+      </c>
+      <c r="S18" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="T18" s="9"/>
+      <c r="U18" s="20"/>
+      <c r="V18" s="20" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="W18" s="20" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="T18" s="20" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="U18" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="19" spans="1:21">
+      <c r="X18" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="19" spans="1:24">
       <c r="A19" s="6" t="s">
         <v>22</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>70</v>
+        <v>61</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>71</v>
+        <v>62</v>
       </c>
       <c r="E19" s="16">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="F19" s="18">
-        <v>320</v>
+        <v>40</v>
       </c>
       <c r="G19" s="18">
         <f t="shared" si="0"/>
-        <v>400</v>
+        <v>50</v>
       </c>
       <c r="H19" s="8" t="s">
-        <v>53</v>
+        <v>26</v>
       </c>
       <c r="I19" s="8" t="s">
-        <v>66</v>
+        <v>36</v>
       </c>
       <c r="J19" s="8" t="s">
-        <v>67</v>
+        <v>37</v>
       </c>
       <c r="K19" s="8" t="s">
-        <v>68</v>
+        <v>38</v>
       </c>
       <c r="L19" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="M19" s="9">
+        <v>0</v>
+      </c>
+      <c r="N19" s="20">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="O19" s="26" t="s">
         <v>57</v>
       </c>
-      <c r="M19" s="9"/>
-      <c r="N19" s="20">
-        <v>144</v>
-      </c>
-      <c r="O19" s="20" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="P19" s="9" t="s">
-        <v>58</v>
-      </c>
-      <c r="Q19" s="9"/>
-      <c r="R19" s="20"/>
-      <c r="S19" s="20" t="str">
+      <c r="P19" s="25">
+        <v>6</v>
+      </c>
+      <c r="Q19" s="25">
+        <f t="shared" si="4"/>
+        <v>864</v>
+      </c>
+      <c r="R19" s="20">
+        <f t="shared" si="5"/>
+        <v>864</v>
+      </c>
+      <c r="S19" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="T19" s="9"/>
+      <c r="U19" s="20"/>
+      <c r="V19" s="20" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="W19" s="20" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="T19" s="20" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="U19" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="20" spans="1:21">
+      <c r="X19" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="20" spans="1:24">
       <c r="A20" s="6" t="s">
         <v>22</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>51</v>
+        <v>70</v>
       </c>
       <c r="D20" s="7" t="s">
-        <v>52</v>
+        <v>71</v>
       </c>
       <c r="E20" s="16">
         <v>0.7</v>
@@ -4664,54 +4910,67 @@
         <v>53</v>
       </c>
       <c r="I20" s="8" t="s">
-        <v>54</v>
+        <v>66</v>
       </c>
       <c r="J20" s="8" t="s">
-        <v>55</v>
+        <v>67</v>
       </c>
       <c r="K20" s="8" t="s">
-        <v>56</v>
+        <v>68</v>
       </c>
       <c r="L20" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="M20" s="9">
+        <v>0</v>
+      </c>
+      <c r="N20" s="20">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="O20" s="26" t="s">
         <v>57</v>
       </c>
-      <c r="M20" s="9"/>
-      <c r="N20" s="20">
-        <v>144</v>
-      </c>
-      <c r="O20" s="20" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="P20" s="9" t="s">
+      <c r="P20" s="25">
+        <v>4</v>
+      </c>
+      <c r="Q20" s="25">
+        <f t="shared" si="4"/>
+        <v>576</v>
+      </c>
+      <c r="R20" s="20">
+        <f t="shared" si="5"/>
+        <v>576</v>
+      </c>
+      <c r="S20" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="Q20" s="9"/>
-      <c r="R20" s="20"/>
-      <c r="S20" s="20" t="str">
+      <c r="T20" s="9"/>
+      <c r="U20" s="20"/>
+      <c r="V20" s="20" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="W20" s="20" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="T20" s="20" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="U20" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="21" spans="1:21">
+      <c r="X20" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="21" spans="1:24" ht="25.5">
       <c r="A21" s="6" t="s">
         <v>22</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C21" s="7" t="s">
-        <v>70</v>
+        <v>51</v>
       </c>
       <c r="D21" s="7" t="s">
-        <v>71</v>
+        <v>52</v>
       </c>
       <c r="E21" s="16">
         <v>0.7</v>
@@ -4727,54 +4986,67 @@
         <v>53</v>
       </c>
       <c r="I21" s="8" t="s">
-        <v>66</v>
+        <v>54</v>
       </c>
       <c r="J21" s="8" t="s">
-        <v>67</v>
+        <v>55</v>
       </c>
       <c r="K21" s="8" t="s">
-        <v>68</v>
+        <v>56</v>
       </c>
       <c r="L21" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="M21" s="9">
+        <v>0</v>
+      </c>
+      <c r="N21" s="20">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="O21" s="26" t="s">
         <v>57</v>
       </c>
-      <c r="M21" s="9"/>
-      <c r="N21" s="20">
+      <c r="P21" s="25">
+        <v>1</v>
+      </c>
+      <c r="Q21" s="25">
+        <f t="shared" si="4"/>
         <v>144</v>
       </c>
-      <c r="O21" s="20" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="P21" s="9" t="s">
+      <c r="R21" s="20">
+        <f t="shared" si="5"/>
+        <v>144</v>
+      </c>
+      <c r="S21" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="Q21" s="9"/>
-      <c r="R21" s="20"/>
-      <c r="S21" s="20" t="str">
+      <c r="T21" s="9"/>
+      <c r="U21" s="20"/>
+      <c r="V21" s="20" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="W21" s="20" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="T21" s="20" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="U21" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="22" spans="1:21">
+      <c r="X21" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="22" spans="1:24">
       <c r="A22" s="6" t="s">
         <v>22</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>51</v>
+        <v>70</v>
       </c>
       <c r="D22" s="7" t="s">
-        <v>52</v>
+        <v>71</v>
       </c>
       <c r="E22" s="16">
         <v>0.7</v>
@@ -4790,117 +5062,143 @@
         <v>53</v>
       </c>
       <c r="I22" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="J22" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="K22" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="L22" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="M22" s="9">
+        <v>0</v>
+      </c>
+      <c r="N22" s="20">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="O22" s="26" t="s">
+        <v>57</v>
+      </c>
+      <c r="P22" s="25">
+        <v>4</v>
+      </c>
+      <c r="Q22" s="25">
+        <f t="shared" si="4"/>
+        <v>576</v>
+      </c>
+      <c r="R22" s="20">
+        <f t="shared" si="5"/>
+        <v>576</v>
+      </c>
+      <c r="S22" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="T22" s="9"/>
+      <c r="U22" s="20"/>
+      <c r="V22" s="20" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="W22" s="20" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="X22" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="23" spans="1:24" ht="25.5">
+      <c r="A23" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B23" s="7" t="s">
+        <v>133</v>
+      </c>
+      <c r="C23" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="D23" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="E23" s="16">
+        <v>0.7</v>
+      </c>
+      <c r="F23" s="18">
+        <v>320</v>
+      </c>
+      <c r="G23" s="18">
+        <f t="shared" si="0"/>
+        <v>400</v>
+      </c>
+      <c r="H23" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="I23" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="J22" s="8" t="s">
+      <c r="J23" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="K22" s="8" t="s">
+      <c r="K23" s="8" t="s">
         <v>56</v>
-      </c>
-      <c r="L22" s="9" t="s">
-        <v>57</v>
-      </c>
-      <c r="M22" s="9"/>
-      <c r="N22" s="20">
-        <v>144</v>
-      </c>
-      <c r="O22" s="20" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="P22" s="9" t="s">
-        <v>58</v>
-      </c>
-      <c r="Q22" s="9"/>
-      <c r="R22" s="20"/>
-      <c r="S22" s="20" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="T22" s="20" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="U22" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="23" spans="1:21">
-      <c r="A23" s="6" t="s">
-        <v>80</v>
-      </c>
-      <c r="B23" s="7" t="s">
-        <v>134</v>
-      </c>
-      <c r="C23" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="D23" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="E23" s="16">
-        <v>0</v>
-      </c>
-      <c r="F23" s="18">
-        <v>80</v>
-      </c>
-      <c r="G23" s="18">
-        <f t="shared" si="0"/>
-        <v>100</v>
-      </c>
-      <c r="H23" s="8" t="s">
-        <v>26</v>
-      </c>
-      <c r="I23" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="J23" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="K23" s="8" t="s">
-        <v>29</v>
       </c>
       <c r="L23" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="M23" s="9"/>
+      <c r="M23" s="9">
+        <v>0</v>
+      </c>
       <c r="N23" s="20">
-        <v>72</v>
-      </c>
-      <c r="O23" s="20" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="P23" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="Q23" s="9"/>
-      <c r="R23" s="20"/>
-      <c r="S23" s="20" t="str">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="O23" s="26" t="s">
+        <v>57</v>
+      </c>
+      <c r="P23" s="25">
+        <v>2</v>
+      </c>
+      <c r="Q23" s="25">
+        <f t="shared" si="4"/>
+        <v>288</v>
+      </c>
+      <c r="R23" s="20">
+        <f t="shared" si="5"/>
+        <v>288</v>
+      </c>
+      <c r="S23" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="T23" s="9"/>
+      <c r="U23" s="20"/>
+      <c r="V23" s="20" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="W23" s="20" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="T23" s="20" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="U23" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="24" spans="1:21">
+      <c r="X23" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="24" spans="1:24">
       <c r="A24" s="6" t="s">
         <v>80</v>
       </c>
       <c r="B24" s="7" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C24" s="7" t="s">
-        <v>136</v>
+        <v>24</v>
       </c>
       <c r="D24" s="7" t="s">
-        <v>137</v>
+        <v>25</v>
       </c>
       <c r="E24" s="16">
         <v>0</v>
@@ -4913,16 +5211,16 @@
         <v>100</v>
       </c>
       <c r="H24" s="8" t="s">
-        <v>42</v>
+        <v>26</v>
       </c>
       <c r="I24" s="8" t="s">
-        <v>115</v>
+        <v>27</v>
       </c>
       <c r="J24" s="8" t="s">
-        <v>116</v>
+        <v>28</v>
       </c>
       <c r="K24" s="8" t="s">
-        <v>117</v>
+        <v>29</v>
       </c>
       <c r="L24" s="9" t="s">
         <v>30</v>
@@ -4931,102 +5229,108 @@
       <c r="N24" s="20">
         <v>72</v>
       </c>
-      <c r="O24" s="20" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="P24" s="9" t="s">
+      <c r="O24" s="25"/>
+      <c r="P24" s="25"/>
+      <c r="Q24" s="25"/>
+      <c r="R24" s="20" t="str">
+        <f t="shared" ref="R24:R37" si="9">IF(OR(M24="",N24=""),"",M24*N24)</f>
+        <v/>
+      </c>
+      <c r="S24" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="Q24" s="9"/>
-      <c r="R24" s="20"/>
-      <c r="S24" s="20" t="str">
+      <c r="T24" s="9"/>
+      <c r="U24" s="20"/>
+      <c r="V24" s="20" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="W24" s="20" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="T24" s="20" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="U24" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="25" spans="1:21">
+      <c r="X24" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="25" spans="1:24" ht="25.5">
       <c r="A25" s="6" t="s">
         <v>80</v>
       </c>
       <c r="B25" s="7" t="s">
-        <v>83</v>
+        <v>135</v>
       </c>
       <c r="C25" s="7" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="D25" s="7" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="E25" s="16">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="F25" s="18">
-        <v>320</v>
+        <v>80</v>
       </c>
       <c r="G25" s="18">
         <f t="shared" si="0"/>
-        <v>400</v>
+        <v>100</v>
       </c>
       <c r="H25" s="8" t="s">
-        <v>53</v>
+        <v>42</v>
       </c>
       <c r="I25" s="8" t="s">
-        <v>66</v>
+        <v>115</v>
       </c>
       <c r="J25" s="8" t="s">
-        <v>67</v>
+        <v>116</v>
       </c>
       <c r="K25" s="8" t="s">
-        <v>68</v>
+        <v>117</v>
       </c>
       <c r="L25" s="9" t="s">
-        <v>57</v>
+        <v>30</v>
       </c>
       <c r="M25" s="9"/>
       <c r="N25" s="20">
-        <v>144</v>
-      </c>
-      <c r="O25" s="20" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="P25" s="9" t="s">
-        <v>58</v>
-      </c>
-      <c r="Q25" s="9"/>
-      <c r="R25" s="20"/>
-      <c r="S25" s="20" t="str">
+        <v>72</v>
+      </c>
+      <c r="O25" s="25"/>
+      <c r="P25" s="25"/>
+      <c r="Q25" s="25"/>
+      <c r="R25" s="20" t="str">
+        <f t="shared" si="9"/>
+        <v/>
+      </c>
+      <c r="S25" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="T25" s="9"/>
+      <c r="U25" s="20"/>
+      <c r="V25" s="20" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="W25" s="20" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="T25" s="20" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="U25" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="26" spans="1:21">
+      <c r="X25" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="26" spans="1:24">
       <c r="A26" s="6" t="s">
         <v>80</v>
       </c>
       <c r="B26" s="7" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C26" s="7" t="s">
-        <v>51</v>
+        <v>138</v>
       </c>
       <c r="D26" s="7" t="s">
-        <v>52</v>
+        <v>139</v>
       </c>
       <c r="E26" s="16">
         <v>0.7</v>
@@ -5042,13 +5346,13 @@
         <v>53</v>
       </c>
       <c r="I26" s="8" t="s">
-        <v>54</v>
+        <v>66</v>
       </c>
       <c r="J26" s="8" t="s">
-        <v>55</v>
+        <v>67</v>
       </c>
       <c r="K26" s="8" t="s">
-        <v>56</v>
+        <v>68</v>
       </c>
       <c r="L26" s="9" t="s">
         <v>57</v>
@@ -5057,39 +5361,42 @@
       <c r="N26" s="20">
         <v>144</v>
       </c>
-      <c r="O26" s="20" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="P26" s="9" t="s">
+      <c r="O26" s="25"/>
+      <c r="P26" s="25"/>
+      <c r="Q26" s="25"/>
+      <c r="R26" s="20" t="str">
+        <f t="shared" si="9"/>
+        <v/>
+      </c>
+      <c r="S26" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="Q26" s="9"/>
-      <c r="R26" s="20"/>
-      <c r="S26" s="20" t="str">
+      <c r="T26" s="9"/>
+      <c r="U26" s="20"/>
+      <c r="V26" s="20" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="W26" s="20" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="T26" s="20" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="U26" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="27" spans="1:21">
+      <c r="X26" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="27" spans="1:24" ht="25.5">
       <c r="A27" s="6" t="s">
         <v>80</v>
       </c>
       <c r="B27" s="7" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="C27" s="7" t="s">
-        <v>70</v>
+        <v>51</v>
       </c>
       <c r="D27" s="7" t="s">
-        <v>71</v>
+        <v>52</v>
       </c>
       <c r="E27" s="16">
         <v>0.7</v>
@@ -5105,13 +5412,13 @@
         <v>53</v>
       </c>
       <c r="I27" s="8" t="s">
-        <v>66</v>
+        <v>54</v>
       </c>
       <c r="J27" s="8" t="s">
-        <v>67</v>
+        <v>55</v>
       </c>
       <c r="K27" s="8" t="s">
-        <v>68</v>
+        <v>56</v>
       </c>
       <c r="L27" s="9" t="s">
         <v>57</v>
@@ -5120,165 +5427,174 @@
       <c r="N27" s="20">
         <v>144</v>
       </c>
-      <c r="O27" s="20" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="P27" s="9" t="s">
+      <c r="O27" s="25"/>
+      <c r="P27" s="25"/>
+      <c r="Q27" s="25"/>
+      <c r="R27" s="20" t="str">
+        <f t="shared" si="9"/>
+        <v/>
+      </c>
+      <c r="S27" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="Q27" s="9"/>
-      <c r="R27" s="20"/>
-      <c r="S27" s="20" t="str">
+      <c r="T27" s="9"/>
+      <c r="U27" s="20"/>
+      <c r="V27" s="20" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="W27" s="20" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="T27" s="20" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="U27" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="28" spans="1:21">
+      <c r="X27" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="28" spans="1:24">
       <c r="A28" s="6" t="s">
         <v>80</v>
       </c>
       <c r="B28" s="7" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="C28" s="7" t="s">
-        <v>140</v>
+        <v>70</v>
       </c>
       <c r="D28" s="7" t="s">
-        <v>141</v>
+        <v>71</v>
       </c>
       <c r="E28" s="16">
-        <v>0.85</v>
+        <v>0.7</v>
       </c>
       <c r="F28" s="18">
-        <v>160</v>
+        <v>320</v>
       </c>
       <c r="G28" s="18">
         <f t="shared" si="0"/>
-        <v>200</v>
+        <v>400</v>
       </c>
       <c r="H28" s="8" t="s">
-        <v>142</v>
+        <v>53</v>
       </c>
       <c r="I28" s="8" t="s">
-        <v>143</v>
+        <v>66</v>
       </c>
       <c r="J28" s="8" t="s">
-        <v>144</v>
+        <v>67</v>
       </c>
       <c r="K28" s="8" t="s">
-        <v>145</v>
+        <v>68</v>
       </c>
       <c r="L28" s="9" t="s">
-        <v>30</v>
+        <v>57</v>
       </c>
       <c r="M28" s="9"/>
       <c r="N28" s="20">
-        <v>72</v>
-      </c>
-      <c r="O28" s="20" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="P28" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="Q28" s="9"/>
-      <c r="R28" s="20"/>
-      <c r="S28" s="20" t="str">
+        <v>144</v>
+      </c>
+      <c r="O28" s="25"/>
+      <c r="P28" s="25"/>
+      <c r="Q28" s="25"/>
+      <c r="R28" s="20" t="str">
+        <f t="shared" si="9"/>
+        <v/>
+      </c>
+      <c r="S28" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="T28" s="9"/>
+      <c r="U28" s="20"/>
+      <c r="V28" s="20" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="W28" s="20" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="T28" s="20" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="U28" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="29" spans="1:21">
+      <c r="X28" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="29" spans="1:24">
       <c r="A29" s="6" t="s">
         <v>80</v>
       </c>
       <c r="B29" s="7" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C29" s="7" t="s">
-        <v>70</v>
+        <v>140</v>
       </c>
       <c r="D29" s="7" t="s">
-        <v>71</v>
+        <v>141</v>
       </c>
       <c r="E29" s="16">
-        <v>0.7</v>
+        <v>0.85</v>
       </c>
       <c r="F29" s="18">
-        <v>320</v>
+        <v>160</v>
       </c>
       <c r="G29" s="18">
         <f t="shared" si="0"/>
-        <v>400</v>
+        <v>200</v>
       </c>
       <c r="H29" s="8" t="s">
-        <v>53</v>
+        <v>142</v>
       </c>
       <c r="I29" s="8" t="s">
-        <v>66</v>
+        <v>143</v>
       </c>
       <c r="J29" s="8" t="s">
-        <v>67</v>
+        <v>144</v>
       </c>
       <c r="K29" s="8" t="s">
-        <v>68</v>
+        <v>145</v>
       </c>
       <c r="L29" s="9" t="s">
-        <v>57</v>
+        <v>30</v>
       </c>
       <c r="M29" s="9"/>
       <c r="N29" s="20">
-        <v>144</v>
-      </c>
-      <c r="O29" s="20" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="P29" s="9" t="s">
-        <v>58</v>
-      </c>
-      <c r="Q29" s="9"/>
-      <c r="R29" s="20"/>
-      <c r="S29" s="20" t="str">
+        <v>72</v>
+      </c>
+      <c r="O29" s="25"/>
+      <c r="P29" s="25"/>
+      <c r="Q29" s="25"/>
+      <c r="R29" s="20" t="str">
+        <f t="shared" si="9"/>
+        <v/>
+      </c>
+      <c r="S29" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="T29" s="9"/>
+      <c r="U29" s="20"/>
+      <c r="V29" s="20" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="W29" s="20" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="T29" s="20" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="U29" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="30" spans="1:21">
+      <c r="X29" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="30" spans="1:24">
       <c r="A30" s="6" t="s">
         <v>80</v>
       </c>
       <c r="B30" s="7" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C30" s="7" t="s">
-        <v>51</v>
+        <v>70</v>
       </c>
       <c r="D30" s="7" t="s">
-        <v>52</v>
+        <v>71</v>
       </c>
       <c r="E30" s="16">
         <v>0.7</v>
@@ -5294,13 +5610,13 @@
         <v>53</v>
       </c>
       <c r="I30" s="8" t="s">
-        <v>54</v>
+        <v>66</v>
       </c>
       <c r="J30" s="8" t="s">
-        <v>55</v>
+        <v>67</v>
       </c>
       <c r="K30" s="8" t="s">
-        <v>56</v>
+        <v>68</v>
       </c>
       <c r="L30" s="9" t="s">
         <v>57</v>
@@ -5309,409 +5625,497 @@
       <c r="N30" s="20">
         <v>144</v>
       </c>
-      <c r="O30" s="20" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="P30" s="9" t="s">
+      <c r="O30" s="25"/>
+      <c r="P30" s="25"/>
+      <c r="Q30" s="25"/>
+      <c r="R30" s="20" t="str">
+        <f t="shared" si="9"/>
+        <v/>
+      </c>
+      <c r="S30" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="Q30" s="9"/>
-      <c r="R30" s="20"/>
-      <c r="S30" s="20" t="str">
+      <c r="T30" s="9"/>
+      <c r="U30" s="20"/>
+      <c r="V30" s="20" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="W30" s="20" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="T30" s="20" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="U30" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="31" spans="1:21" ht="28">
+      <c r="X30" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="31" spans="1:24" ht="25.5">
       <c r="A31" s="6" t="s">
         <v>80</v>
       </c>
       <c r="B31" s="7" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C31" s="7" t="s">
-        <v>40</v>
+        <v>51</v>
       </c>
       <c r="D31" s="7" t="s">
-        <v>41</v>
+        <v>52</v>
       </c>
       <c r="E31" s="16">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="F31" s="18">
-        <v>80</v>
+        <v>320</v>
       </c>
       <c r="G31" s="18">
-        <f>ROUND(F31/0.8,0)</f>
-        <v>100</v>
+        <f t="shared" si="0"/>
+        <v>400</v>
       </c>
       <c r="H31" s="8" t="s">
-        <v>42</v>
+        <v>53</v>
       </c>
       <c r="I31" s="8" t="s">
-        <v>43</v>
+        <v>54</v>
       </c>
       <c r="J31" s="8" t="s">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="K31" s="8" t="s">
-        <v>45</v>
+        <v>56</v>
       </c>
       <c r="L31" s="9" t="s">
-        <v>30</v>
+        <v>57</v>
       </c>
       <c r="M31" s="9"/>
       <c r="N31" s="20">
-        <v>72</v>
-      </c>
-      <c r="O31" s="20" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="P31" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="Q31" s="9"/>
-      <c r="R31" s="20"/>
-      <c r="S31" s="20" t="str">
+        <v>144</v>
+      </c>
+      <c r="O31" s="25"/>
+      <c r="P31" s="25"/>
+      <c r="Q31" s="25"/>
+      <c r="R31" s="20" t="str">
+        <f t="shared" si="9"/>
+        <v/>
+      </c>
+      <c r="S31" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="T31" s="9"/>
+      <c r="U31" s="20"/>
+      <c r="V31" s="20" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="W31" s="20" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="T31" s="20" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="U31" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="32" spans="1:21">
+      <c r="X31" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="32" spans="1:24" ht="25.5">
       <c r="A32" s="6" t="s">
         <v>80</v>
       </c>
       <c r="B32" s="7" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C32" s="7" t="s">
-        <v>70</v>
+        <v>40</v>
       </c>
       <c r="D32" s="7" t="s">
-        <v>71</v>
+        <v>41</v>
       </c>
       <c r="E32" s="16">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="F32" s="18">
-        <v>320</v>
+        <v>80</v>
       </c>
       <c r="G32" s="18">
-        <f t="shared" si="0"/>
-        <v>400</v>
+        <f>ROUND(F32/0.8,0)</f>
+        <v>100</v>
       </c>
       <c r="H32" s="8" t="s">
-        <v>53</v>
+        <v>42</v>
       </c>
       <c r="I32" s="8" t="s">
-        <v>66</v>
+        <v>43</v>
       </c>
       <c r="J32" s="8" t="s">
-        <v>67</v>
+        <v>44</v>
       </c>
       <c r="K32" s="8" t="s">
-        <v>68</v>
+        <v>45</v>
       </c>
       <c r="L32" s="9" t="s">
-        <v>57</v>
+        <v>30</v>
       </c>
       <c r="M32" s="9"/>
       <c r="N32" s="20">
-        <v>144</v>
-      </c>
-      <c r="O32" s="20" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="P32" s="9" t="s">
-        <v>58</v>
-      </c>
-      <c r="Q32" s="9"/>
-      <c r="R32" s="20"/>
-      <c r="S32" s="20" t="str">
+        <v>72</v>
+      </c>
+      <c r="O32" s="25"/>
+      <c r="P32" s="25"/>
+      <c r="Q32" s="25"/>
+      <c r="R32" s="20" t="str">
+        <f t="shared" si="9"/>
+        <v/>
+      </c>
+      <c r="S32" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="T32" s="9"/>
+      <c r="U32" s="20"/>
+      <c r="V32" s="20" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="W32" s="20" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="T32" s="20" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="U32" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="33" spans="1:21" ht="28">
+      <c r="X32" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="33" spans="1:24">
       <c r="A33" s="6" t="s">
         <v>80</v>
       </c>
       <c r="B33" s="7" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C33" s="7" t="s">
-        <v>40</v>
+        <v>70</v>
       </c>
       <c r="D33" s="7" t="s">
-        <v>41</v>
+        <v>71</v>
       </c>
       <c r="E33" s="16">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="F33" s="18">
-        <v>80</v>
+        <v>320</v>
       </c>
       <c r="G33" s="18">
         <f t="shared" si="0"/>
-        <v>100</v>
+        <v>400</v>
       </c>
       <c r="H33" s="8" t="s">
-        <v>42</v>
+        <v>53</v>
       </c>
       <c r="I33" s="8" t="s">
-        <v>43</v>
+        <v>66</v>
       </c>
       <c r="J33" s="8" t="s">
-        <v>44</v>
+        <v>67</v>
       </c>
       <c r="K33" s="8" t="s">
-        <v>45</v>
+        <v>68</v>
       </c>
       <c r="L33" s="9" t="s">
-        <v>30</v>
+        <v>57</v>
       </c>
       <c r="M33" s="9"/>
       <c r="N33" s="20">
-        <v>72</v>
-      </c>
-      <c r="O33" s="20" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="P33" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="Q33" s="9"/>
-      <c r="R33" s="20"/>
-      <c r="S33" s="20" t="str">
+        <v>144</v>
+      </c>
+      <c r="O33" s="25"/>
+      <c r="P33" s="25"/>
+      <c r="Q33" s="25"/>
+      <c r="R33" s="20" t="str">
+        <f t="shared" si="9"/>
+        <v/>
+      </c>
+      <c r="S33" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="T33" s="9"/>
+      <c r="U33" s="20"/>
+      <c r="V33" s="20" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="W33" s="20" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="T33" s="20" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="U33" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="34" spans="1:21">
+      <c r="X33" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="34" spans="1:24" ht="25.5">
       <c r="A34" s="6" t="s">
         <v>80</v>
       </c>
       <c r="B34" s="7" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C34" s="7" t="s">
-        <v>70</v>
+        <v>40</v>
       </c>
       <c r="D34" s="7" t="s">
-        <v>71</v>
+        <v>41</v>
       </c>
       <c r="E34" s="16">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="F34" s="18">
-        <v>320</v>
+        <v>80</v>
       </c>
       <c r="G34" s="18">
         <f t="shared" si="0"/>
-        <v>400</v>
+        <v>100</v>
       </c>
       <c r="H34" s="8" t="s">
-        <v>53</v>
+        <v>42</v>
       </c>
       <c r="I34" s="8" t="s">
-        <v>66</v>
+        <v>43</v>
       </c>
       <c r="J34" s="8" t="s">
-        <v>67</v>
+        <v>44</v>
       </c>
       <c r="K34" s="8" t="s">
-        <v>68</v>
+        <v>45</v>
       </c>
       <c r="L34" s="9" t="s">
-        <v>57</v>
+        <v>30</v>
       </c>
       <c r="M34" s="9"/>
       <c r="N34" s="20">
-        <v>144</v>
-      </c>
-      <c r="O34" s="20" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="P34" s="9" t="s">
-        <v>58</v>
-      </c>
-      <c r="Q34" s="9"/>
-      <c r="R34" s="20"/>
-      <c r="S34" s="20" t="str">
+        <v>72</v>
+      </c>
+      <c r="O34" s="25"/>
+      <c r="P34" s="25"/>
+      <c r="Q34" s="25"/>
+      <c r="R34" s="20" t="str">
+        <f t="shared" si="9"/>
+        <v/>
+      </c>
+      <c r="S34" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="T34" s="9"/>
+      <c r="U34" s="20"/>
+      <c r="V34" s="20" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="W34" s="20" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="T34" s="20" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="U34" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="35" spans="1:21">
+      <c r="X34" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="35" spans="1:24">
       <c r="A35" s="6" t="s">
         <v>80</v>
       </c>
       <c r="B35" s="7" t="s">
-        <v>146</v>
+        <v>96</v>
       </c>
       <c r="C35" s="7" t="s">
-        <v>136</v>
+        <v>70</v>
       </c>
       <c r="D35" s="7" t="s">
-        <v>137</v>
+        <v>71</v>
       </c>
       <c r="E35" s="16">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="F35" s="18">
-        <v>80</v>
+        <v>320</v>
       </c>
       <c r="G35" s="18">
         <f t="shared" si="0"/>
-        <v>100</v>
+        <v>400</v>
       </c>
       <c r="H35" s="8" t="s">
-        <v>42</v>
+        <v>53</v>
       </c>
       <c r="I35" s="8" t="s">
-        <v>115</v>
+        <v>66</v>
       </c>
       <c r="J35" s="8" t="s">
-        <v>116</v>
+        <v>67</v>
       </c>
       <c r="K35" s="8" t="s">
-        <v>117</v>
+        <v>68</v>
       </c>
       <c r="L35" s="9" t="s">
-        <v>30</v>
+        <v>57</v>
       </c>
       <c r="M35" s="9"/>
       <c r="N35" s="20">
+        <v>144</v>
+      </c>
+      <c r="O35" s="25"/>
+      <c r="P35" s="25"/>
+      <c r="Q35" s="25"/>
+      <c r="R35" s="20" t="str">
+        <f t="shared" si="9"/>
+        <v/>
+      </c>
+      <c r="S35" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="T35" s="9"/>
+      <c r="U35" s="20"/>
+      <c r="V35" s="20" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="W35" s="20" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="X35" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="36" spans="1:24" ht="25.5">
+      <c r="A36" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="B36" s="7" t="s">
+        <v>146</v>
+      </c>
+      <c r="C36" s="7" t="s">
+        <v>136</v>
+      </c>
+      <c r="D36" s="7" t="s">
+        <v>137</v>
+      </c>
+      <c r="E36" s="16">
+        <v>0</v>
+      </c>
+      <c r="F36" s="18">
+        <v>80</v>
+      </c>
+      <c r="G36" s="18">
+        <f t="shared" si="0"/>
+        <v>100</v>
+      </c>
+      <c r="H36" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="I36" s="8" t="s">
+        <v>115</v>
+      </c>
+      <c r="J36" s="8" t="s">
+        <v>116</v>
+      </c>
+      <c r="K36" s="8" t="s">
+        <v>117</v>
+      </c>
+      <c r="L36" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="M36" s="9"/>
+      <c r="N36" s="20">
         <v>72</v>
       </c>
-      <c r="O35" s="20" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="P35" s="9" t="s">
+      <c r="O36" s="25"/>
+      <c r="P36" s="25"/>
+      <c r="Q36" s="25"/>
+      <c r="R36" s="20" t="str">
+        <f t="shared" si="9"/>
+        <v/>
+      </c>
+      <c r="S36" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="Q35" s="9"/>
-      <c r="R35" s="20"/>
-      <c r="S35" s="20" t="str">
+      <c r="T36" s="9"/>
+      <c r="U36" s="20"/>
+      <c r="V36" s="20" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="W36" s="20" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="T35" s="20" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="U35" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="36" spans="1:21">
-      <c r="A36" s="11" t="s">
+      <c r="X36" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="37" spans="1:24" ht="25.5">
+      <c r="A37" s="11" t="s">
         <v>80</v>
       </c>
-      <c r="B36" s="12" t="s">
+      <c r="B37" s="12" t="s">
         <v>99</v>
       </c>
-      <c r="C36" s="12" t="s">
+      <c r="C37" s="12" t="s">
         <v>147</v>
       </c>
-      <c r="D36" s="12" t="s">
+      <c r="D37" s="12" t="s">
         <v>148</v>
       </c>
-      <c r="E36" s="17">
+      <c r="E37" s="17">
         <v>0.7</v>
       </c>
-      <c r="F36" s="19">
+      <c r="F37" s="19">
         <v>320</v>
       </c>
-      <c r="G36" s="19">
+      <c r="G37" s="19">
         <f t="shared" si="0"/>
         <v>400</v>
       </c>
-      <c r="H36" s="13" t="s">
+      <c r="H37" s="13" t="s">
         <v>53</v>
       </c>
-      <c r="I36" s="13" t="s">
+      <c r="I37" s="13" t="s">
         <v>54</v>
       </c>
-      <c r="J36" s="13" t="s">
+      <c r="J37" s="13" t="s">
         <v>55</v>
       </c>
-      <c r="K36" s="13" t="s">
+      <c r="K37" s="13" t="s">
         <v>56</v>
       </c>
-      <c r="L36" s="14" t="s">
+      <c r="L37" s="14" t="s">
         <v>57</v>
       </c>
-      <c r="M36" s="14"/>
-      <c r="N36" s="21">
+      <c r="M37" s="14"/>
+      <c r="N37" s="21">
         <v>144</v>
       </c>
-      <c r="O36" s="21" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="P36" s="14" t="s">
+      <c r="O37" s="25"/>
+      <c r="P37" s="25"/>
+      <c r="Q37" s="25"/>
+      <c r="R37" s="21" t="str">
+        <f t="shared" si="9"/>
+        <v/>
+      </c>
+      <c r="S37" s="14" t="s">
         <v>58</v>
       </c>
-      <c r="Q36" s="14"/>
-      <c r="R36" s="21"/>
-      <c r="S36" s="21" t="str">
+      <c r="T37" s="14"/>
+      <c r="U37" s="21"/>
+      <c r="V37" s="21" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="W37" s="21" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="T36" s="21" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="U36" s="15" t="s">
+      <c r="X37" s="15" t="s">
         <v>32</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:U1"/>
+    <mergeCell ref="A1:X1"/>
   </mergeCells>
+  <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -5719,7 +6123,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:H12"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
+  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
     <col min="2" max="3" width="16" customWidth="1"/>
@@ -5727,19 +6131,19 @@
     <col min="6" max="8" width="34" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="21">
-      <c r="A1" s="26" t="s">
+    <row r="1" spans="1:8" ht="20.25">
+      <c r="A1" s="28" t="s">
         <v>149</v>
       </c>
-      <c r="B1" s="26"/>
-      <c r="C1" s="26"/>
-      <c r="D1" s="26"/>
-      <c r="E1" s="26"/>
-      <c r="F1" s="26"/>
-      <c r="G1" s="26"/>
-      <c r="H1" s="26"/>
-    </row>
-    <row r="2" spans="1:8" ht="32">
+      <c r="B1" s="28"/>
+      <c r="C1" s="28"/>
+      <c r="D1" s="28"/>
+      <c r="E1" s="28"/>
+      <c r="F1" s="28"/>
+      <c r="G1" s="28"/>
+      <c r="H1" s="28"/>
+    </row>
+    <row r="2" spans="1:8" ht="30">
       <c r="A2" s="1" t="s">
         <v>150</v>
       </c>
@@ -5765,7 +6169,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="30">
+    <row r="3" spans="1:8" ht="28.5">
       <c r="A3" s="2" t="s">
         <v>71</v>
       </c>
@@ -5792,7 +6196,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="30">
+    <row r="4" spans="1:8" ht="28.5">
       <c r="A4" s="2" t="s">
         <v>160</v>
       </c>
@@ -5819,7 +6223,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="15">
+    <row r="5" spans="1:8">
       <c r="A5" s="2" t="s">
         <v>124</v>
       </c>
@@ -5846,7 +6250,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="15">
+    <row r="6" spans="1:8">
       <c r="A6" s="2" t="s">
         <v>62</v>
       </c>
@@ -5873,7 +6277,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="15">
+    <row r="7" spans="1:8">
       <c r="A7" s="2" t="s">
         <v>24</v>
       </c>
@@ -5900,7 +6304,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="15">
+    <row r="8" spans="1:8">
       <c r="A8" s="2" t="s">
         <v>109</v>
       </c>
@@ -5927,7 +6331,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="15">
+    <row r="9" spans="1:8">
       <c r="A9" s="2" t="s">
         <v>172</v>
       </c>
@@ -5954,7 +6358,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="30">
+    <row r="10" spans="1:8" ht="28.5">
       <c r="A10" s="2" t="s">
         <v>176</v>
       </c>
@@ -5981,7 +6385,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="15">
+    <row r="11" spans="1:8">
       <c r="A11" s="2" t="s">
         <v>178</v>
       </c>
@@ -6008,7 +6412,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="15">
+    <row r="12" spans="1:8">
       <c r="A12" s="2" t="s">
         <v>181</v>
       </c>

</xml_diff>

<commit_message>
Added Liam's alpha design file, completed existing luminaires for building A
</commit_message>
<xml_diff>
--- a/Building A B Lighting New.xlsx
+++ b/Building A B Lighting New.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lsen906\Documents\Alpha_Design_17\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D764F81-86BA-4BC3-A730-A242110B5A33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEF100CD-F807-4868-89E7-1A2A637BF8B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Building A" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="891" uniqueCount="188">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="895" uniqueCount="192">
   <si>
     <t>Building A — Lighting Place Schedule</t>
   </si>
@@ -598,7 +598,19 @@
     <t>Existing Qty (2)</t>
   </si>
   <si>
-    <t>Existing W each (2)</t>
+    <t>Existing Illuminance (lx)</t>
+  </si>
+  <si>
+    <t>Slope: 181 Flat: 237</t>
+  </si>
+  <si>
+    <t>Slope: 267 Flat: 226</t>
+  </si>
+  <si>
+    <t>Existing W</t>
+  </si>
+  <si>
+    <t>Existing W (2)</t>
   </si>
 </sst>
 </file>
@@ -756,7 +768,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -840,11 +852,144 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="3" fillId="6" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="18">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
@@ -1011,7 +1156,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:X36"/>
+  <dimension ref="A1:Y36"/>
   <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="2" width="10" customWidth="1"/>
@@ -1025,13 +1170,13 @@
     <col min="12" max="12" width="22" customWidth="1"/>
     <col min="13" max="14" width="12" customWidth="1"/>
     <col min="15" max="15" width="14" customWidth="1"/>
-    <col min="16" max="16" width="24" customWidth="1"/>
-    <col min="17" max="18" width="12" customWidth="1"/>
-    <col min="19" max="20" width="14" customWidth="1"/>
-    <col min="21" max="21" width="16" customWidth="1"/>
+    <col min="16" max="16" width="8.375" customWidth="1"/>
+    <col min="17" max="19" width="12" customWidth="1"/>
+    <col min="20" max="21" width="14" customWidth="1"/>
+    <col min="22" max="22" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" ht="20.25">
+    <row r="1" spans="1:25" ht="20.25">
       <c r="A1" s="27" t="s">
         <v>0</v>
       </c>
@@ -1055,8 +1200,9 @@
       <c r="S1" s="27"/>
       <c r="T1" s="27"/>
       <c r="U1" s="27"/>
-    </row>
-    <row r="2" spans="1:24" ht="45">
+      <c r="V1" s="27"/>
+    </row>
+    <row r="2" spans="1:25" ht="45">
       <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
@@ -1111,26 +1257,29 @@
       <c r="R2" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="S2" s="4" t="s">
+      <c r="S2" s="29" t="s">
+        <v>187</v>
+      </c>
+      <c r="T2" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="T2" s="4" t="s">
+      <c r="U2" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="U2" s="4" t="s">
+      <c r="V2" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="V2" s="4" t="s">
+      <c r="W2" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="W2" s="4" t="s">
+      <c r="X2" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="X2" s="5" t="s">
+      <c r="Y2" s="5" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:24" ht="25.5">
+    <row r="3" spans="1:25" ht="25.5">
       <c r="A3" s="6" t="s">
         <v>22</v>
       </c>
@@ -1181,24 +1330,27 @@
         <f>IF(OR(M3="",N3=""),"",M3*N3)</f>
         <v>72</v>
       </c>
-      <c r="S3" s="9" t="s">
+      <c r="S3" s="30" t="s">
+        <v>189</v>
+      </c>
+      <c r="T3" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="T3" s="9"/>
-      <c r="U3" s="20"/>
-      <c r="V3" s="20" t="str">
-        <f>IF(OR(T3="",U3=""),"",T3*U3)</f>
-        <v/>
-      </c>
+      <c r="U3" s="9"/>
+      <c r="V3" s="20"/>
       <c r="W3" s="20" t="str">
-        <f t="shared" ref="W3:W36" si="1">IF(OR(R3="",V3=""),"",R3-V3)</f>
-        <v/>
-      </c>
-      <c r="X3" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="4" spans="1:24" ht="25.5">
+        <f>IF(OR(U3="",V3=""),"",U3*V3)</f>
+        <v/>
+      </c>
+      <c r="X3" s="20" t="str">
+        <f t="shared" ref="X3:X36" si="1">IF(OR(R3="",W3=""),"",R3-W3)</f>
+        <v/>
+      </c>
+      <c r="Y3" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="4" spans="1:25" ht="25.5">
       <c r="A4" s="6" t="s">
         <v>22</v>
       </c>
@@ -1256,24 +1408,27 @@
         <f>IF(OR(M4="",N4=""),"",M4*N4+Q4)</f>
         <v>288</v>
       </c>
-      <c r="S4" s="9" t="s">
+      <c r="S4" s="30">
+        <v>503</v>
+      </c>
+      <c r="T4" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="T4" s="9"/>
-      <c r="U4" s="20"/>
-      <c r="V4" s="20" t="str">
-        <f>IF(OR(T4="",U4=""),"",T4*U4)</f>
-        <v/>
-      </c>
+      <c r="U4" s="9"/>
+      <c r="V4" s="20"/>
       <c r="W4" s="20" t="str">
+        <f>IF(OR(U4="",V4=""),"",U4*V4)</f>
+        <v/>
+      </c>
+      <c r="X4" s="20" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="X4" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="5" spans="1:24" ht="25.5">
+      <c r="Y4" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="5" spans="1:25" ht="25.5">
       <c r="A5" s="6" t="s">
         <v>22</v>
       </c>
@@ -1324,24 +1479,27 @@
         <f t="shared" ref="R5:R35" si="2">IF(OR(M5="",N5=""),"",M5*N5)</f>
         <v>72</v>
       </c>
-      <c r="S5" s="9" t="s">
+      <c r="S5" s="30">
+        <v>209</v>
+      </c>
+      <c r="T5" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="T5" s="9"/>
-      <c r="U5" s="20"/>
-      <c r="V5" s="20" t="str">
-        <f t="shared" ref="V5:V36" si="3">IF(OR(T5="",U5=""),"",T5*U5)</f>
-        <v/>
-      </c>
+      <c r="U5" s="9"/>
+      <c r="V5" s="20"/>
       <c r="W5" s="20" t="str">
+        <f t="shared" ref="W5:W36" si="3">IF(OR(U5="",V5=""),"",U5*V5)</f>
+        <v/>
+      </c>
+      <c r="X5" s="20" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="X5" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="6" spans="1:24" ht="25.5">
+      <c r="Y5" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="6" spans="1:25" ht="25.5">
       <c r="A6" s="6" t="s">
         <v>22</v>
       </c>
@@ -1392,24 +1550,27 @@
         <f t="shared" si="2"/>
         <v>72</v>
       </c>
-      <c r="S6" s="9" t="s">
+      <c r="S6" s="30">
+        <v>209</v>
+      </c>
+      <c r="T6" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="T6" s="9"/>
-      <c r="U6" s="20"/>
-      <c r="V6" s="20" t="str">
+      <c r="U6" s="9"/>
+      <c r="V6" s="20"/>
+      <c r="W6" s="20" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="W6" s="20" t="str">
+      <c r="X6" s="20" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="X6" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="7" spans="1:24" ht="25.5">
+      <c r="Y6" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="7" spans="1:25" ht="25.5">
       <c r="A7" s="6" t="s">
         <v>22</v>
       </c>
@@ -1460,24 +1621,27 @@
         <f t="shared" si="2"/>
         <v>72</v>
       </c>
-      <c r="S7" s="9" t="s">
+      <c r="S7" s="30">
+        <v>183</v>
+      </c>
+      <c r="T7" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="T7" s="9"/>
-      <c r="U7" s="20"/>
-      <c r="V7" s="20" t="str">
+      <c r="U7" s="9"/>
+      <c r="V7" s="20"/>
+      <c r="W7" s="20" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="W7" s="20" t="str">
+      <c r="X7" s="20" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="X7" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="8" spans="1:24" ht="25.5">
+      <c r="Y7" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="8" spans="1:25" ht="25.5">
       <c r="A8" s="6" t="s">
         <v>22</v>
       </c>
@@ -1528,24 +1692,27 @@
         <f t="shared" si="2"/>
         <v>288</v>
       </c>
-      <c r="S8" s="9" t="s">
+      <c r="S8" s="30">
+        <v>625</v>
+      </c>
+      <c r="T8" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="T8" s="9"/>
-      <c r="U8" s="20"/>
-      <c r="V8" s="20" t="str">
+      <c r="U8" s="9"/>
+      <c r="V8" s="20"/>
+      <c r="W8" s="20" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="W8" s="20" t="str">
+      <c r="X8" s="20" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="X8" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="9" spans="1:24" ht="25.5">
+      <c r="Y8" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="9" spans="1:25" ht="25.5">
       <c r="A9" s="6" t="s">
         <v>22</v>
       </c>
@@ -1596,24 +1763,27 @@
         <f t="shared" si="2"/>
         <v>288</v>
       </c>
-      <c r="S9" s="9" t="s">
+      <c r="S9" s="30">
+        <v>644</v>
+      </c>
+      <c r="T9" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="T9" s="9"/>
-      <c r="U9" s="20"/>
-      <c r="V9" s="20" t="str">
+      <c r="U9" s="9"/>
+      <c r="V9" s="20"/>
+      <c r="W9" s="20" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="W9" s="20" t="str">
+      <c r="X9" s="20" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="X9" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="10" spans="1:24" ht="25.5">
+      <c r="Y9" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="10" spans="1:25" ht="25.5">
       <c r="A10" s="6" t="s">
         <v>22</v>
       </c>
@@ -1671,24 +1841,27 @@
         <f>IF(OR(M10="",N10=""),"",M10*N10+Q10)</f>
         <v>432</v>
       </c>
-      <c r="S10" s="9" t="s">
+      <c r="S10" s="30">
+        <v>373</v>
+      </c>
+      <c r="T10" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="T10" s="9"/>
-      <c r="U10" s="20"/>
-      <c r="V10" s="20" t="str">
+      <c r="U10" s="9"/>
+      <c r="V10" s="20"/>
+      <c r="W10" s="20" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="W10" s="20" t="str">
+      <c r="X10" s="20" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="X10" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="11" spans="1:24" ht="25.5">
+      <c r="Y10" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="11" spans="1:25" ht="25.5">
       <c r="A11" s="6" t="s">
         <v>22</v>
       </c>
@@ -1739,24 +1912,26 @@
         <f t="shared" si="2"/>
         <v>288</v>
       </c>
-      <c r="S11" s="9" t="s">
+      <c r="S11" s="30">
+        <v>615</v>
+      </c>
+      <c r="T11" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="T11" s="9"/>
-      <c r="U11" s="20"/>
-      <c r="V11" s="20" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
+      <c r="V11" s="20"/>
       <c r="W11" s="20" t="str">
+        <f>IF(OR(U12="",V11=""),"",U12*V11)</f>
+        <v/>
+      </c>
+      <c r="X11" s="20" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="X11" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="12" spans="1:24" ht="25.5">
+      <c r="Y11" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="12" spans="1:25" ht="25.5">
       <c r="A12" s="6" t="s">
         <v>22</v>
       </c>
@@ -1807,24 +1982,27 @@
         <f t="shared" si="2"/>
         <v>576</v>
       </c>
-      <c r="S12" s="9" t="s">
+      <c r="S12" s="30">
+        <v>836</v>
+      </c>
+      <c r="T12" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="T12" s="9"/>
-      <c r="U12" s="20"/>
-      <c r="V12" s="20" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="W12" s="20" t="str">
+      <c r="U12" s="9"/>
+      <c r="V12" s="20"/>
+      <c r="W12" s="20" t="e">
+        <f>IF(OR(#REF!="",V12=""),"",#REF!*V12)</f>
+        <v>#REF!</v>
+      </c>
+      <c r="X12" s="20" t="e">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="X12" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="13" spans="1:24" ht="25.5">
+        <v>#REF!</v>
+      </c>
+      <c r="Y12" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="13" spans="1:25" ht="25.5">
       <c r="A13" s="6" t="s">
         <v>22</v>
       </c>
@@ -1875,24 +2053,27 @@
         <f t="shared" si="2"/>
         <v>576</v>
       </c>
-      <c r="S13" s="9" t="s">
+      <c r="S13" s="30">
+        <v>743</v>
+      </c>
+      <c r="T13" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="T13" s="9"/>
-      <c r="U13" s="20"/>
-      <c r="V13" s="20" t="str">
+      <c r="U13" s="9"/>
+      <c r="V13" s="20"/>
+      <c r="W13" s="20" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="W13" s="20" t="str">
+      <c r="X13" s="20" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="X13" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="14" spans="1:24" ht="25.5">
+      <c r="Y13" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="14" spans="1:25" ht="25.5">
       <c r="A14" s="6" t="s">
         <v>22</v>
       </c>
@@ -1943,24 +2124,27 @@
         <f t="shared" si="2"/>
         <v>864</v>
       </c>
-      <c r="S14" s="9" t="s">
+      <c r="S14" s="30">
+        <v>1088</v>
+      </c>
+      <c r="T14" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="T14" s="9"/>
-      <c r="U14" s="20"/>
-      <c r="V14" s="20" t="str">
+      <c r="U14" s="9"/>
+      <c r="V14" s="20"/>
+      <c r="W14" s="20" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="W14" s="20" t="str">
+      <c r="X14" s="20" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="X14" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="15" spans="1:24" ht="25.5">
+      <c r="Y14" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="15" spans="1:25" ht="25.5">
       <c r="A15" s="6" t="s">
         <v>22</v>
       </c>
@@ -2011,24 +2195,27 @@
         <f t="shared" si="2"/>
         <v>432</v>
       </c>
-      <c r="S15" s="9" t="s">
+      <c r="S15" s="30">
+        <v>743</v>
+      </c>
+      <c r="T15" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="T15" s="9"/>
-      <c r="U15" s="20"/>
-      <c r="V15" s="20" t="str">
+      <c r="U15" s="9"/>
+      <c r="V15" s="20"/>
+      <c r="W15" s="20" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="W15" s="20" t="str">
+      <c r="X15" s="20" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="X15" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="16" spans="1:24" ht="25.5">
+      <c r="Y15" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="16" spans="1:25" ht="25.5">
       <c r="A16" s="6" t="s">
         <v>22</v>
       </c>
@@ -2079,24 +2266,27 @@
         <f t="shared" si="2"/>
         <v>432</v>
       </c>
-      <c r="S16" s="9" t="s">
+      <c r="S16" s="30">
+        <v>954</v>
+      </c>
+      <c r="T16" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="T16" s="9"/>
-      <c r="U16" s="20"/>
-      <c r="V16" s="20" t="str">
+      <c r="U16" s="9"/>
+      <c r="V16" s="20"/>
+      <c r="W16" s="20" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="W16" s="20" t="str">
+      <c r="X16" s="20" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="X16" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="17" spans="1:24" ht="25.5">
+      <c r="Y16" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="17" spans="1:25" ht="25.5">
       <c r="A17" s="6" t="s">
         <v>80</v>
       </c>
@@ -2147,24 +2337,27 @@
         <f t="shared" si="2"/>
         <v>72</v>
       </c>
-      <c r="S17" s="9" t="s">
+      <c r="S17" s="30">
+        <v>150</v>
+      </c>
+      <c r="T17" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="T17" s="9"/>
-      <c r="U17" s="20"/>
-      <c r="V17" s="20" t="str">
+      <c r="U17" s="9"/>
+      <c r="V17" s="20"/>
+      <c r="W17" s="20" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="W17" s="20" t="str">
+      <c r="X17" s="20" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="X17" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="18" spans="1:24" ht="25.5">
+      <c r="Y17" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="18" spans="1:25" ht="25.5">
       <c r="A18" s="6" t="s">
         <v>80</v>
       </c>
@@ -2215,24 +2408,27 @@
         <f t="shared" si="2"/>
         <v>288</v>
       </c>
-      <c r="S18" s="9" t="s">
+      <c r="S18" s="30">
+        <v>140</v>
+      </c>
+      <c r="T18" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="T18" s="9"/>
-      <c r="U18" s="20"/>
-      <c r="V18" s="20" t="str">
+      <c r="U18" s="9"/>
+      <c r="V18" s="20"/>
+      <c r="W18" s="20" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="W18" s="20" t="str">
+      <c r="X18" s="20" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="X18" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="19" spans="1:24" ht="25.5">
+      <c r="Y18" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="19" spans="1:25" ht="25.5">
       <c r="A19" s="6" t="s">
         <v>80</v>
       </c>
@@ -2283,24 +2479,27 @@
         <f t="shared" si="2"/>
         <v>288</v>
       </c>
-      <c r="S19" s="9" t="s">
+      <c r="S19" s="30">
+        <v>331</v>
+      </c>
+      <c r="T19" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="T19" s="9"/>
-      <c r="U19" s="20"/>
-      <c r="V19" s="20" t="str">
+      <c r="U19" s="9"/>
+      <c r="V19" s="20"/>
+      <c r="W19" s="20" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="W19" s="20" t="str">
+      <c r="X19" s="20" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="X19" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="20" spans="1:24" ht="25.5">
+      <c r="Y19" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="20" spans="1:25" ht="25.5">
       <c r="A20" s="6" t="s">
         <v>80</v>
       </c>
@@ -2351,24 +2550,27 @@
         <f t="shared" si="2"/>
         <v>1008</v>
       </c>
-      <c r="S20" s="9" t="s">
+      <c r="S20" s="30">
+        <v>470</v>
+      </c>
+      <c r="T20" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="T20" s="9"/>
-      <c r="U20" s="20"/>
-      <c r="V20" s="20" t="str">
+      <c r="U20" s="9"/>
+      <c r="V20" s="20"/>
+      <c r="W20" s="20" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="W20" s="20" t="str">
+      <c r="X20" s="20" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="X20" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="21" spans="1:24" ht="25.5">
+      <c r="Y20" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="21" spans="1:25" ht="25.5">
       <c r="A21" s="6" t="s">
         <v>80</v>
       </c>
@@ -2419,24 +2621,27 @@
         <f t="shared" si="2"/>
         <v>72</v>
       </c>
-      <c r="S21" s="9" t="s">
+      <c r="S21" s="30">
+        <v>181</v>
+      </c>
+      <c r="T21" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="T21" s="9"/>
-      <c r="U21" s="20"/>
-      <c r="V21" s="20" t="str">
+      <c r="U21" s="9"/>
+      <c r="V21" s="20"/>
+      <c r="W21" s="20" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="W21" s="20" t="str">
+      <c r="X21" s="20" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="X21" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="22" spans="1:24" ht="25.5">
+      <c r="Y21" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="22" spans="1:25" ht="25.5">
       <c r="A22" s="6" t="s">
         <v>80</v>
       </c>
@@ -2487,24 +2692,27 @@
         <f t="shared" si="2"/>
         <v>144</v>
       </c>
-      <c r="S22" s="9" t="s">
+      <c r="S22" s="30">
+        <v>269</v>
+      </c>
+      <c r="T22" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="T22" s="9"/>
-      <c r="U22" s="20"/>
-      <c r="V22" s="20" t="str">
+      <c r="U22" s="9"/>
+      <c r="V22" s="20"/>
+      <c r="W22" s="20" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="W22" s="20" t="str">
+      <c r="X22" s="20" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="X22" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="23" spans="1:24" ht="25.5">
+      <c r="Y22" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="23" spans="1:25" ht="25.5">
       <c r="A23" s="6" t="s">
         <v>80</v>
       </c>
@@ -2555,24 +2763,27 @@
         <f t="shared" si="2"/>
         <v>864</v>
       </c>
-      <c r="S23" s="9" t="s">
+      <c r="S23" s="30">
+        <v>516</v>
+      </c>
+      <c r="T23" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="T23" s="9"/>
-      <c r="U23" s="20"/>
-      <c r="V23" s="20" t="str">
+      <c r="U23" s="9"/>
+      <c r="V23" s="20"/>
+      <c r="W23" s="20" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="W23" s="20" t="str">
+      <c r="X23" s="20" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="X23" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="24" spans="1:24" ht="25.5">
+      <c r="Y23" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="24" spans="1:25" ht="25.5">
       <c r="A24" s="6" t="s">
         <v>80</v>
       </c>
@@ -2623,24 +2834,27 @@
         <f t="shared" si="2"/>
         <v>576</v>
       </c>
-      <c r="S24" s="9" t="s">
+      <c r="S24" s="30">
+        <v>458</v>
+      </c>
+      <c r="T24" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="T24" s="9"/>
-      <c r="U24" s="20"/>
-      <c r="V24" s="20" t="str">
+      <c r="U24" s="9"/>
+      <c r="V24" s="20"/>
+      <c r="W24" s="20" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="W24" s="20" t="str">
+      <c r="X24" s="20" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="X24" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="25" spans="1:24" ht="25.5">
+      <c r="Y24" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="25" spans="1:25" ht="25.5">
       <c r="A25" s="6" t="s">
         <v>80</v>
       </c>
@@ -2691,24 +2905,27 @@
         <f t="shared" si="2"/>
         <v>576</v>
       </c>
-      <c r="S25" s="9" t="s">
+      <c r="S25" s="30">
+        <v>422</v>
+      </c>
+      <c r="T25" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="T25" s="9"/>
-      <c r="U25" s="20"/>
-      <c r="V25" s="20" t="str">
+      <c r="U25" s="9"/>
+      <c r="V25" s="20"/>
+      <c r="W25" s="20" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="W25" s="20" t="str">
+      <c r="X25" s="20" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="X25" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="26" spans="1:24" ht="25.5">
+      <c r="Y25" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="26" spans="1:25" ht="25.5">
       <c r="A26" s="6" t="s">
         <v>80</v>
       </c>
@@ -2759,24 +2976,27 @@
         <f t="shared" si="2"/>
         <v>1152</v>
       </c>
-      <c r="S26" s="9" t="s">
+      <c r="S26" s="30">
+        <v>455</v>
+      </c>
+      <c r="T26" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="T26" s="9"/>
-      <c r="U26" s="20"/>
-      <c r="V26" s="20" t="str">
+      <c r="U26" s="9"/>
+      <c r="V26" s="20"/>
+      <c r="W26" s="20" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="W26" s="20" t="str">
+      <c r="X26" s="20" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="X26" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="27" spans="1:24" ht="25.5">
+      <c r="Y26" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="27" spans="1:25" ht="25.5">
       <c r="A27" s="6" t="s">
         <v>80</v>
       </c>
@@ -2827,24 +3047,27 @@
         <f t="shared" si="2"/>
         <v>576</v>
       </c>
-      <c r="S27" s="9" t="s">
+      <c r="S27" s="30">
+        <v>133</v>
+      </c>
+      <c r="T27" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="T27" s="9"/>
-      <c r="U27" s="20"/>
-      <c r="V27" s="20" t="str">
+      <c r="U27" s="9"/>
+      <c r="V27" s="20"/>
+      <c r="W27" s="20" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="W27" s="20" t="str">
+      <c r="X27" s="20" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="X27" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="28" spans="1:24" ht="25.5">
+      <c r="Y27" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="28" spans="1:25" ht="25.5">
       <c r="A28" s="6" t="s">
         <v>80</v>
       </c>
@@ -2895,24 +3118,27 @@
         <f t="shared" si="2"/>
         <v>1152</v>
       </c>
-      <c r="S28" s="9" t="s">
+      <c r="S28" s="30">
+        <v>435</v>
+      </c>
+      <c r="T28" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="T28" s="9"/>
-      <c r="U28" s="20"/>
-      <c r="V28" s="20" t="str">
+      <c r="U28" s="9"/>
+      <c r="V28" s="20"/>
+      <c r="W28" s="20" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="W28" s="20" t="str">
+      <c r="X28" s="20" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="X28" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="29" spans="1:24" ht="25.5">
+      <c r="Y28" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="29" spans="1:25" ht="25.5">
       <c r="A29" s="6" t="s">
         <v>80</v>
       </c>
@@ -2963,24 +3189,27 @@
         <f t="shared" si="2"/>
         <v>72</v>
       </c>
-      <c r="S29" s="9" t="s">
+      <c r="S29" s="30">
+        <v>118</v>
+      </c>
+      <c r="T29" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="T29" s="9"/>
-      <c r="U29" s="20"/>
-      <c r="V29" s="20" t="str">
+      <c r="U29" s="9"/>
+      <c r="V29" s="20"/>
+      <c r="W29" s="20" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="W29" s="20" t="str">
+      <c r="X29" s="20" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="X29" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="30" spans="1:24" ht="25.5">
+      <c r="Y29" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="30" spans="1:25" ht="25.5">
       <c r="A30" s="6" t="s">
         <v>80</v>
       </c>
@@ -3031,24 +3260,27 @@
         <f t="shared" si="2"/>
         <v>576</v>
       </c>
-      <c r="S30" s="9" t="s">
+      <c r="S30" s="30">
+        <v>416</v>
+      </c>
+      <c r="T30" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="T30" s="9"/>
-      <c r="U30" s="20"/>
-      <c r="V30" s="20" t="str">
+      <c r="U30" s="9"/>
+      <c r="V30" s="20"/>
+      <c r="W30" s="20" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="W30" s="20" t="str">
+      <c r="X30" s="20" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="X30" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="31" spans="1:24" ht="25.5">
+      <c r="Y30" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="31" spans="1:25" ht="25.5">
       <c r="A31" s="6" t="s">
         <v>80</v>
       </c>
@@ -3099,24 +3331,27 @@
         <f t="shared" si="2"/>
         <v>576</v>
       </c>
-      <c r="S31" s="9" t="s">
+      <c r="S31" s="30">
+        <v>419</v>
+      </c>
+      <c r="T31" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="T31" s="9"/>
-      <c r="U31" s="20"/>
-      <c r="V31" s="20" t="str">
+      <c r="U31" s="9"/>
+      <c r="V31" s="20"/>
+      <c r="W31" s="20" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="W31" s="20" t="str">
+      <c r="X31" s="20" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="X31" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="32" spans="1:24" ht="25.5">
+      <c r="Y31" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="32" spans="1:25" ht="25.5">
       <c r="A32" s="6" t="s">
         <v>80</v>
       </c>
@@ -3167,24 +3402,27 @@
         <f t="shared" si="2"/>
         <v>576</v>
       </c>
-      <c r="S32" s="9" t="s">
+      <c r="S32" s="30">
+        <v>400</v>
+      </c>
+      <c r="T32" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="T32" s="9"/>
-      <c r="U32" s="20"/>
-      <c r="V32" s="20" t="str">
+      <c r="U32" s="9"/>
+      <c r="V32" s="20"/>
+      <c r="W32" s="20" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="W32" s="20" t="str">
+      <c r="X32" s="20" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="X32" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="33" spans="1:24" ht="25.5">
+      <c r="Y32" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="33" spans="1:25" ht="25.5">
       <c r="A33" s="6" t="s">
         <v>80</v>
       </c>
@@ -3235,24 +3473,27 @@
         <f t="shared" si="2"/>
         <v>72</v>
       </c>
-      <c r="S33" s="9" t="s">
+      <c r="S33" s="30">
+        <v>140</v>
+      </c>
+      <c r="T33" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="T33" s="9"/>
-      <c r="U33" s="20"/>
-      <c r="V33" s="20" t="str">
+      <c r="U33" s="9"/>
+      <c r="V33" s="20"/>
+      <c r="W33" s="20" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="W33" s="20" t="str">
+      <c r="X33" s="20" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="X33" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="34" spans="1:24" ht="25.5">
+      <c r="Y33" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="34" spans="1:25" ht="25.5">
       <c r="A34" s="6" t="s">
         <v>80</v>
       </c>
@@ -3303,24 +3544,27 @@
         <f t="shared" si="2"/>
         <v>72</v>
       </c>
-      <c r="S34" s="9" t="s">
+      <c r="S34" s="30">
+        <v>140</v>
+      </c>
+      <c r="T34" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="T34" s="9"/>
-      <c r="U34" s="20"/>
-      <c r="V34" s="20" t="str">
+      <c r="U34" s="9"/>
+      <c r="V34" s="20"/>
+      <c r="W34" s="20" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="W34" s="20" t="str">
+      <c r="X34" s="20" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="X34" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="35" spans="1:24" ht="25.5">
+      <c r="Y34" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="35" spans="1:25" ht="25.5">
       <c r="A35" s="6" t="s">
         <v>80</v>
       </c>
@@ -3371,24 +3615,27 @@
         <f t="shared" si="2"/>
         <v>432</v>
       </c>
-      <c r="S35" s="9" t="s">
+      <c r="S35" s="30">
+        <v>405</v>
+      </c>
+      <c r="T35" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="T35" s="9"/>
-      <c r="U35" s="20"/>
-      <c r="V35" s="20" t="str">
+      <c r="U35" s="9"/>
+      <c r="V35" s="20"/>
+      <c r="W35" s="20" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="W35" s="20" t="str">
+      <c r="X35" s="20" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="X35" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="36" spans="1:24" ht="25.5">
+      <c r="Y35" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="36" spans="1:25" ht="25.5">
       <c r="A36" s="11" t="s">
         <v>80</v>
       </c>
@@ -3439,34 +3686,46 @@
         <f>IF(OR(M36="",N36=""),"",M36*N36)</f>
         <v>576</v>
       </c>
-      <c r="S36" s="14" t="s">
+      <c r="S36" s="30">
+        <v>392</v>
+      </c>
+      <c r="T36" s="14" t="s">
         <v>58</v>
       </c>
-      <c r="T36" s="14"/>
-      <c r="U36" s="21"/>
-      <c r="V36" s="21" t="str">
+      <c r="U36" s="14"/>
+      <c r="V36" s="21"/>
+      <c r="W36" s="21" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="W36" s="21" t="str">
+      <c r="X36" s="21" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="X36" s="15" t="s">
+      <c r="Y36" s="15" t="s">
         <v>32</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:U1"/>
+    <mergeCell ref="A1:V1"/>
   </mergeCells>
+  <conditionalFormatting sqref="S4:S36">
+    <cfRule type="expression" dxfId="3" priority="1">
+      <formula>$S4&lt;$F4</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="2" priority="2">
+      <formula>$S4&gt;=$F4</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:X37"/>
+  <dimension ref="A1:Y37"/>
   <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="2" width="10" customWidth="1"/>
@@ -3482,14 +3741,14 @@
     <col min="15" max="15" width="14" customWidth="1"/>
     <col min="16" max="16" width="15.625" customWidth="1"/>
     <col min="17" max="17" width="12" customWidth="1"/>
-    <col min="18" max="18" width="14" customWidth="1"/>
-    <col min="19" max="19" width="24" customWidth="1"/>
-    <col min="20" max="21" width="12" customWidth="1"/>
-    <col min="22" max="23" width="14" customWidth="1"/>
-    <col min="24" max="24" width="16" customWidth="1"/>
+    <col min="18" max="19" width="14" customWidth="1"/>
+    <col min="20" max="20" width="24" customWidth="1"/>
+    <col min="21" max="22" width="12" customWidth="1"/>
+    <col min="23" max="24" width="14" customWidth="1"/>
+    <col min="25" max="25" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" ht="20.25">
+    <row r="1" spans="1:25" ht="20.25">
       <c r="A1" s="27" t="s">
         <v>107</v>
       </c>
@@ -3516,8 +3775,9 @@
       <c r="V1" s="27"/>
       <c r="W1" s="27"/>
       <c r="X1" s="27"/>
-    </row>
-    <row r="2" spans="1:24" ht="30">
+      <c r="Y1" s="27"/>
+    </row>
+    <row r="2" spans="1:25" ht="45">
       <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
@@ -3558,7 +3818,7 @@
         <v>13</v>
       </c>
       <c r="N2" s="4" t="s">
-        <v>14</v>
+        <v>190</v>
       </c>
       <c r="O2" s="4" t="s">
         <v>185</v>
@@ -3567,31 +3827,34 @@
         <v>186</v>
       </c>
       <c r="Q2" s="4" t="s">
-        <v>187</v>
+        <v>191</v>
       </c>
       <c r="R2" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="S2" s="4" t="s">
+      <c r="S2" s="29" t="s">
+        <v>187</v>
+      </c>
+      <c r="T2" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="T2" s="4" t="s">
+      <c r="U2" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="U2" s="4" t="s">
+      <c r="V2" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="V2" s="4" t="s">
+      <c r="W2" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="W2" s="4" t="s">
+      <c r="X2" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="X2" s="5" t="s">
+      <c r="Y2" s="5" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:24">
+    <row r="3" spans="1:25" ht="25.5">
       <c r="A3" s="6" t="s">
         <v>22</v>
       </c>
@@ -3650,24 +3913,27 @@
         <f>N3+Q3</f>
         <v>72</v>
       </c>
-      <c r="S3" s="9" t="s">
+      <c r="S3" s="30" t="s">
+        <v>188</v>
+      </c>
+      <c r="T3" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="T3" s="9"/>
-      <c r="U3" s="20"/>
-      <c r="V3" s="20" t="str">
-        <f t="shared" ref="V3:V37" si="1">IF(OR(T3="",U3=""),"",T3*U3)</f>
-        <v/>
-      </c>
+      <c r="U3" s="9"/>
+      <c r="V3" s="20"/>
       <c r="W3" s="20" t="str">
-        <f t="shared" ref="W3:W37" si="2">IF(OR(R3="",V3=""),"",R3-V3)</f>
-        <v/>
-      </c>
-      <c r="X3" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="4" spans="1:24">
+        <f t="shared" ref="W3:W37" si="1">IF(OR(U3="",V3=""),"",U3*V3)</f>
+        <v/>
+      </c>
+      <c r="X3" s="20" t="str">
+        <f t="shared" ref="X3:X37" si="2">IF(OR(R3="",W3=""),"",R3-W3)</f>
+        <v/>
+      </c>
+      <c r="Y3" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="4" spans="1:25">
       <c r="A4" s="6" t="s">
         <v>22</v>
       </c>
@@ -3726,24 +3992,27 @@
         <f t="shared" ref="R4:R23" si="5">N4+Q4</f>
         <v>864</v>
       </c>
-      <c r="S4" s="9" t="s">
+      <c r="S4" s="30">
+        <v>380</v>
+      </c>
+      <c r="T4" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="T4" s="9"/>
-      <c r="U4" s="20"/>
-      <c r="V4" s="20" t="str">
+      <c r="U4" s="9"/>
+      <c r="V4" s="20"/>
+      <c r="W4" s="20" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="W4" s="20" t="str">
+      <c r="X4" s="20" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="X4" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="5" spans="1:24" ht="25.5">
+      <c r="Y4" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="5" spans="1:25" ht="25.5">
       <c r="A5" s="6" t="s">
         <v>22</v>
       </c>
@@ -3802,24 +4071,27 @@
         <f t="shared" si="5"/>
         <v>144</v>
       </c>
-      <c r="S5" s="9" t="s">
+      <c r="S5" s="30">
+        <v>325</v>
+      </c>
+      <c r="T5" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="T5" s="9"/>
-      <c r="U5" s="20"/>
-      <c r="V5" s="20" t="str">
+      <c r="U5" s="9"/>
+      <c r="V5" s="20"/>
+      <c r="W5" s="20" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="W5" s="20" t="str">
+      <c r="X5" s="20" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="X5" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="6" spans="1:24" ht="25.5">
+      <c r="Y5" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="6" spans="1:25" ht="25.5">
       <c r="A6" s="6" t="s">
         <v>22</v>
       </c>
@@ -3878,24 +4150,27 @@
         <f t="shared" si="5"/>
         <v>72</v>
       </c>
-      <c r="S6" s="9" t="s">
+      <c r="S6" s="30">
+        <v>205</v>
+      </c>
+      <c r="T6" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="T6" s="9"/>
-      <c r="U6" s="20"/>
-      <c r="V6" s="20" t="str">
+      <c r="U6" s="9"/>
+      <c r="V6" s="20"/>
+      <c r="W6" s="20" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="W6" s="20" t="str">
+      <c r="X6" s="20" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="X6" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="7" spans="1:24" ht="25.5">
+      <c r="Y6" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="7" spans="1:25" ht="25.5">
       <c r="A7" s="6" t="s">
         <v>22</v>
       </c>
@@ -3954,24 +4229,27 @@
         <f t="shared" si="5"/>
         <v>72</v>
       </c>
-      <c r="S7" s="9" t="s">
+      <c r="S7" s="30">
+        <v>201</v>
+      </c>
+      <c r="T7" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="T7" s="9"/>
-      <c r="U7" s="20"/>
-      <c r="V7" s="20" t="str">
+      <c r="U7" s="9"/>
+      <c r="V7" s="20"/>
+      <c r="W7" s="20" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="W7" s="20" t="str">
+      <c r="X7" s="20" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="X7" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="8" spans="1:24" ht="25.5">
+      <c r="Y7" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="8" spans="1:25" ht="25.5">
       <c r="A8" s="6" t="s">
         <v>22</v>
       </c>
@@ -4030,24 +4308,27 @@
         <f t="shared" si="5"/>
         <v>72</v>
       </c>
-      <c r="S8" s="9" t="s">
+      <c r="S8" s="30">
+        <v>186</v>
+      </c>
+      <c r="T8" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="T8" s="9"/>
-      <c r="U8" s="20"/>
-      <c r="V8" s="20" t="str">
+      <c r="U8" s="9"/>
+      <c r="V8" s="20"/>
+      <c r="W8" s="20" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="W8" s="20" t="str">
+      <c r="X8" s="20" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="X8" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="9" spans="1:24" ht="25.5">
+      <c r="Y8" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="9" spans="1:25" ht="25.5">
       <c r="A9" s="6" t="s">
         <v>22</v>
       </c>
@@ -4106,24 +4387,27 @@
         <f t="shared" si="5"/>
         <v>72</v>
       </c>
-      <c r="S9" s="9" t="s">
+      <c r="S9" s="30">
+        <v>187</v>
+      </c>
+      <c r="T9" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="T9" s="9"/>
-      <c r="U9" s="20"/>
-      <c r="V9" s="20" t="str">
+      <c r="U9" s="9"/>
+      <c r="V9" s="20"/>
+      <c r="W9" s="20" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="W9" s="20" t="str">
+      <c r="X9" s="20" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="X9" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="10" spans="1:24">
+      <c r="Y9" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="10" spans="1:25">
       <c r="A10" s="6" t="s">
         <v>22</v>
       </c>
@@ -4182,24 +4466,27 @@
         <f t="shared" si="5"/>
         <v>576</v>
       </c>
-      <c r="S10" s="9" t="s">
+      <c r="S10" s="30">
+        <v>753</v>
+      </c>
+      <c r="T10" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="T10" s="9"/>
-      <c r="U10" s="20"/>
-      <c r="V10" s="20" t="str">
+      <c r="U10" s="9"/>
+      <c r="V10" s="20"/>
+      <c r="W10" s="20" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="W10" s="20" t="str">
+      <c r="X10" s="20" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="X10" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="11" spans="1:24">
+      <c r="Y10" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="11" spans="1:25">
       <c r="A11" s="6" t="s">
         <v>22</v>
       </c>
@@ -4258,24 +4545,27 @@
         <f>N11+Q11</f>
         <v>288</v>
       </c>
-      <c r="S11" s="9" t="s">
+      <c r="S11" s="30">
+        <v>801</v>
+      </c>
+      <c r="T11" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="T11" s="9"/>
-      <c r="U11" s="20"/>
-      <c r="V11" s="20" t="str">
-        <f t="shared" ref="V11" si="7">IF(OR(T11="",U11=""),"",T11*U11)</f>
-        <v/>
-      </c>
+      <c r="U11" s="9"/>
+      <c r="V11" s="20"/>
       <c r="W11" s="20" t="str">
-        <f t="shared" ref="W11" si="8">IF(OR(R11="",V11=""),"",R11-V11)</f>
-        <v/>
-      </c>
-      <c r="X11" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="12" spans="1:24">
+        <f t="shared" ref="W11" si="7">IF(OR(U11="",V11=""),"",U11*V11)</f>
+        <v/>
+      </c>
+      <c r="X11" s="20" t="str">
+        <f t="shared" ref="X11" si="8">IF(OR(R11="",W11=""),"",R11-W11)</f>
+        <v/>
+      </c>
+      <c r="Y11" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="12" spans="1:25">
       <c r="A12" s="6" t="s">
         <v>22</v>
       </c>
@@ -4334,24 +4624,27 @@
         <f t="shared" si="5"/>
         <v>864</v>
       </c>
-      <c r="S12" s="9" t="s">
+      <c r="S12" s="30">
+        <v>1107</v>
+      </c>
+      <c r="T12" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="T12" s="9"/>
-      <c r="U12" s="20"/>
-      <c r="V12" s="20" t="str">
+      <c r="U12" s="9"/>
+      <c r="V12" s="20"/>
+      <c r="W12" s="20" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="W12" s="20" t="str">
+      <c r="X12" s="20" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="X12" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="13" spans="1:24">
+      <c r="Y12" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="13" spans="1:25">
       <c r="A13" s="6" t="s">
         <v>22</v>
       </c>
@@ -4410,24 +4703,27 @@
         <f t="shared" si="5"/>
         <v>288</v>
       </c>
-      <c r="S13" s="9" t="s">
+      <c r="S13" s="30">
+        <v>740</v>
+      </c>
+      <c r="T13" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="T13" s="9"/>
-      <c r="U13" s="20"/>
-      <c r="V13" s="20" t="str">
+      <c r="U13" s="9"/>
+      <c r="V13" s="20"/>
+      <c r="W13" s="20" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="W13" s="20" t="str">
+      <c r="X13" s="20" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="X13" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="14" spans="1:24" ht="25.5">
+      <c r="Y13" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="14" spans="1:25" ht="25.5">
       <c r="A14" s="6" t="s">
         <v>22</v>
       </c>
@@ -4486,24 +4782,27 @@
         <f t="shared" si="5"/>
         <v>432</v>
       </c>
-      <c r="S14" s="9" t="s">
+      <c r="S14" s="30">
+        <v>865</v>
+      </c>
+      <c r="T14" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="T14" s="9"/>
-      <c r="U14" s="20"/>
-      <c r="V14" s="20" t="str">
+      <c r="U14" s="9"/>
+      <c r="V14" s="20"/>
+      <c r="W14" s="20" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="W14" s="20" t="str">
+      <c r="X14" s="20" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="X14" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="15" spans="1:24">
+      <c r="Y14" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="15" spans="1:25">
       <c r="A15" s="6" t="s">
         <v>22</v>
       </c>
@@ -4562,24 +4861,27 @@
         <f t="shared" si="5"/>
         <v>288</v>
       </c>
-      <c r="S15" s="9" t="s">
+      <c r="S15" s="30">
+        <v>403</v>
+      </c>
+      <c r="T15" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="T15" s="9"/>
-      <c r="U15" s="20"/>
-      <c r="V15" s="20" t="str">
+      <c r="U15" s="9"/>
+      <c r="V15" s="20"/>
+      <c r="W15" s="20" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="W15" s="20" t="str">
+      <c r="X15" s="20" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="X15" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="16" spans="1:24" ht="25.5">
+      <c r="Y15" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="16" spans="1:25" ht="25.5">
       <c r="A16" s="6" t="s">
         <v>22</v>
       </c>
@@ -4638,24 +4940,27 @@
         <f t="shared" si="5"/>
         <v>144</v>
       </c>
-      <c r="S16" s="9" t="s">
+      <c r="S16" s="30">
+        <v>403</v>
+      </c>
+      <c r="T16" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="T16" s="9"/>
-      <c r="U16" s="20"/>
-      <c r="V16" s="20" t="str">
+      <c r="U16" s="9"/>
+      <c r="V16" s="20"/>
+      <c r="W16" s="20" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="W16" s="20" t="str">
+      <c r="X16" s="20" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="X16" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="17" spans="1:24" ht="25.5">
+      <c r="Y16" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="17" spans="1:25" ht="25.5">
       <c r="A17" s="6" t="s">
         <v>22</v>
       </c>
@@ -4714,24 +5019,27 @@
         <f t="shared" si="5"/>
         <v>576</v>
       </c>
-      <c r="S17" s="9" t="s">
+      <c r="S17" s="30">
+        <v>1069</v>
+      </c>
+      <c r="T17" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="T17" s="9"/>
-      <c r="U17" s="20"/>
-      <c r="V17" s="20" t="str">
+      <c r="U17" s="9"/>
+      <c r="V17" s="20"/>
+      <c r="W17" s="20" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="W17" s="20" t="str">
+      <c r="X17" s="20" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="X17" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="18" spans="1:24" ht="25.5">
+      <c r="Y17" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="18" spans="1:25" ht="25.5">
       <c r="A18" s="6" t="s">
         <v>22</v>
       </c>
@@ -4790,24 +5098,27 @@
         <f t="shared" si="5"/>
         <v>288</v>
       </c>
-      <c r="S18" s="9" t="s">
+      <c r="S18" s="30">
+        <v>854</v>
+      </c>
+      <c r="T18" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="T18" s="9"/>
-      <c r="U18" s="20"/>
-      <c r="V18" s="20" t="str">
+      <c r="U18" s="9"/>
+      <c r="V18" s="20"/>
+      <c r="W18" s="20" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="W18" s="20" t="str">
+      <c r="X18" s="20" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="X18" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="19" spans="1:24">
+      <c r="Y18" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="19" spans="1:25">
       <c r="A19" s="6" t="s">
         <v>22</v>
       </c>
@@ -4866,24 +5177,27 @@
         <f t="shared" si="5"/>
         <v>864</v>
       </c>
-      <c r="S19" s="9" t="s">
+      <c r="S19" s="30">
+        <v>538</v>
+      </c>
+      <c r="T19" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="T19" s="9"/>
-      <c r="U19" s="20"/>
-      <c r="V19" s="20" t="str">
+      <c r="U19" s="9"/>
+      <c r="V19" s="20"/>
+      <c r="W19" s="20" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="W19" s="20" t="str">
+      <c r="X19" s="20" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="X19" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="20" spans="1:24">
+      <c r="Y19" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="20" spans="1:25">
       <c r="A20" s="6" t="s">
         <v>22</v>
       </c>
@@ -4942,24 +5256,27 @@
         <f t="shared" si="5"/>
         <v>576</v>
       </c>
-      <c r="S20" s="9" t="s">
+      <c r="S20" s="30">
+        <v>1064</v>
+      </c>
+      <c r="T20" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="T20" s="9"/>
-      <c r="U20" s="20"/>
-      <c r="V20" s="20" t="str">
+      <c r="U20" s="9"/>
+      <c r="V20" s="20"/>
+      <c r="W20" s="20" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="W20" s="20" t="str">
+      <c r="X20" s="20" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="X20" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="21" spans="1:24" ht="25.5">
+      <c r="Y20" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="21" spans="1:25" ht="25.5">
       <c r="A21" s="6" t="s">
         <v>22</v>
       </c>
@@ -5018,24 +5335,27 @@
         <f t="shared" si="5"/>
         <v>144</v>
       </c>
-      <c r="S21" s="9" t="s">
+      <c r="S21" s="30">
+        <v>538</v>
+      </c>
+      <c r="T21" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="T21" s="9"/>
-      <c r="U21" s="20"/>
-      <c r="V21" s="20" t="str">
+      <c r="U21" s="9"/>
+      <c r="V21" s="20"/>
+      <c r="W21" s="20" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="W21" s="20" t="str">
+      <c r="X21" s="20" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="X21" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="22" spans="1:24">
+      <c r="Y21" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="22" spans="1:25">
       <c r="A22" s="6" t="s">
         <v>22</v>
       </c>
@@ -5094,24 +5414,27 @@
         <f t="shared" si="5"/>
         <v>576</v>
       </c>
-      <c r="S22" s="9" t="s">
+      <c r="S22" s="30">
+        <v>1133</v>
+      </c>
+      <c r="T22" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="T22" s="9"/>
-      <c r="U22" s="20"/>
-      <c r="V22" s="20" t="str">
+      <c r="U22" s="9"/>
+      <c r="V22" s="20"/>
+      <c r="W22" s="20" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="W22" s="20" t="str">
+      <c r="X22" s="20" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="X22" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="23" spans="1:24" ht="25.5">
+      <c r="Y22" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="23" spans="1:25" ht="25.5">
       <c r="A23" s="6" t="s">
         <v>22</v>
       </c>
@@ -5170,24 +5493,27 @@
         <f t="shared" si="5"/>
         <v>288</v>
       </c>
-      <c r="S23" s="9" t="s">
+      <c r="S23" s="30">
+        <v>900</v>
+      </c>
+      <c r="T23" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="T23" s="9"/>
-      <c r="U23" s="20"/>
-      <c r="V23" s="20" t="str">
+      <c r="U23" s="9"/>
+      <c r="V23" s="20"/>
+      <c r="W23" s="20" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="W23" s="20" t="str">
+      <c r="X23" s="20" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="X23" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="24" spans="1:24">
+      <c r="Y23" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="24" spans="1:25">
       <c r="A24" s="6" t="s">
         <v>80</v>
       </c>
@@ -5236,24 +5562,25 @@
         <f t="shared" ref="R24:R37" si="9">IF(OR(M24="",N24=""),"",M24*N24)</f>
         <v/>
       </c>
-      <c r="S24" s="9" t="s">
+      <c r="S24" s="30"/>
+      <c r="T24" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="T24" s="9"/>
-      <c r="U24" s="20"/>
-      <c r="V24" s="20" t="str">
+      <c r="U24" s="9"/>
+      <c r="V24" s="20"/>
+      <c r="W24" s="20" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="W24" s="20" t="str">
+      <c r="X24" s="20" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="X24" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="25" spans="1:24" ht="25.5">
+      <c r="Y24" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="25" spans="1:25" ht="25.5">
       <c r="A25" s="6" t="s">
         <v>80</v>
       </c>
@@ -5302,24 +5629,25 @@
         <f t="shared" si="9"/>
         <v/>
       </c>
-      <c r="S25" s="9" t="s">
+      <c r="S25" s="30"/>
+      <c r="T25" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="T25" s="9"/>
-      <c r="U25" s="20"/>
-      <c r="V25" s="20" t="str">
+      <c r="U25" s="9"/>
+      <c r="V25" s="20"/>
+      <c r="W25" s="20" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="W25" s="20" t="str">
+      <c r="X25" s="20" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="X25" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="26" spans="1:24">
+      <c r="Y25" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="26" spans="1:25">
       <c r="A26" s="6" t="s">
         <v>80</v>
       </c>
@@ -5368,24 +5696,25 @@
         <f t="shared" si="9"/>
         <v/>
       </c>
-      <c r="S26" s="9" t="s">
+      <c r="S26" s="30"/>
+      <c r="T26" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="T26" s="9"/>
-      <c r="U26" s="20"/>
-      <c r="V26" s="20" t="str">
+      <c r="U26" s="9"/>
+      <c r="V26" s="20"/>
+      <c r="W26" s="20" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="W26" s="20" t="str">
+      <c r="X26" s="20" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="X26" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="27" spans="1:24" ht="25.5">
+      <c r="Y26" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="27" spans="1:25" ht="25.5">
       <c r="A27" s="6" t="s">
         <v>80</v>
       </c>
@@ -5434,24 +5763,25 @@
         <f t="shared" si="9"/>
         <v/>
       </c>
-      <c r="S27" s="9" t="s">
+      <c r="S27" s="30"/>
+      <c r="T27" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="T27" s="9"/>
-      <c r="U27" s="20"/>
-      <c r="V27" s="20" t="str">
+      <c r="U27" s="9"/>
+      <c r="V27" s="20"/>
+      <c r="W27" s="20" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="W27" s="20" t="str">
+      <c r="X27" s="20" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="X27" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="28" spans="1:24">
+      <c r="Y27" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="28" spans="1:25">
       <c r="A28" s="6" t="s">
         <v>80</v>
       </c>
@@ -5500,24 +5830,25 @@
         <f t="shared" si="9"/>
         <v/>
       </c>
-      <c r="S28" s="9" t="s">
+      <c r="S28" s="30"/>
+      <c r="T28" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="T28" s="9"/>
-      <c r="U28" s="20"/>
-      <c r="V28" s="20" t="str">
+      <c r="U28" s="9"/>
+      <c r="V28" s="20"/>
+      <c r="W28" s="20" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="W28" s="20" t="str">
+      <c r="X28" s="20" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="X28" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="29" spans="1:24">
+      <c r="Y28" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="29" spans="1:25">
       <c r="A29" s="6" t="s">
         <v>80</v>
       </c>
@@ -5566,24 +5897,25 @@
         <f t="shared" si="9"/>
         <v/>
       </c>
-      <c r="S29" s="9" t="s">
+      <c r="S29" s="30"/>
+      <c r="T29" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="T29" s="9"/>
-      <c r="U29" s="20"/>
-      <c r="V29" s="20" t="str">
+      <c r="U29" s="9"/>
+      <c r="V29" s="20"/>
+      <c r="W29" s="20" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="W29" s="20" t="str">
+      <c r="X29" s="20" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="X29" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="30" spans="1:24">
+      <c r="Y29" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="30" spans="1:25">
       <c r="A30" s="6" t="s">
         <v>80</v>
       </c>
@@ -5632,24 +5964,25 @@
         <f t="shared" si="9"/>
         <v/>
       </c>
-      <c r="S30" s="9" t="s">
+      <c r="S30" s="30"/>
+      <c r="T30" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="T30" s="9"/>
-      <c r="U30" s="20"/>
-      <c r="V30" s="20" t="str">
+      <c r="U30" s="9"/>
+      <c r="V30" s="20"/>
+      <c r="W30" s="20" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="W30" s="20" t="str">
+      <c r="X30" s="20" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="X30" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="31" spans="1:24" ht="25.5">
+      <c r="Y30" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="31" spans="1:25" ht="25.5">
       <c r="A31" s="6" t="s">
         <v>80</v>
       </c>
@@ -5698,24 +6031,25 @@
         <f t="shared" si="9"/>
         <v/>
       </c>
-      <c r="S31" s="9" t="s">
+      <c r="S31" s="30"/>
+      <c r="T31" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="T31" s="9"/>
-      <c r="U31" s="20"/>
-      <c r="V31" s="20" t="str">
+      <c r="U31" s="9"/>
+      <c r="V31" s="20"/>
+      <c r="W31" s="20" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="W31" s="20" t="str">
+      <c r="X31" s="20" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="X31" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="32" spans="1:24" ht="25.5">
+      <c r="Y31" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="32" spans="1:25" ht="25.5">
       <c r="A32" s="6" t="s">
         <v>80</v>
       </c>
@@ -5764,24 +6098,25 @@
         <f t="shared" si="9"/>
         <v/>
       </c>
-      <c r="S32" s="9" t="s">
+      <c r="S32" s="30"/>
+      <c r="T32" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="T32" s="9"/>
-      <c r="U32" s="20"/>
-      <c r="V32" s="20" t="str">
+      <c r="U32" s="9"/>
+      <c r="V32" s="20"/>
+      <c r="W32" s="20" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="W32" s="20" t="str">
+      <c r="X32" s="20" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="X32" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="33" spans="1:24">
+      <c r="Y32" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="33" spans="1:25">
       <c r="A33" s="6" t="s">
         <v>80</v>
       </c>
@@ -5830,24 +6165,25 @@
         <f t="shared" si="9"/>
         <v/>
       </c>
-      <c r="S33" s="9" t="s">
+      <c r="S33" s="30"/>
+      <c r="T33" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="T33" s="9"/>
-      <c r="U33" s="20"/>
-      <c r="V33" s="20" t="str">
+      <c r="U33" s="9"/>
+      <c r="V33" s="20"/>
+      <c r="W33" s="20" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="W33" s="20" t="str">
+      <c r="X33" s="20" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="X33" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="34" spans="1:24" ht="25.5">
+      <c r="Y33" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="34" spans="1:25" ht="25.5">
       <c r="A34" s="6" t="s">
         <v>80</v>
       </c>
@@ -5896,24 +6232,25 @@
         <f t="shared" si="9"/>
         <v/>
       </c>
-      <c r="S34" s="9" t="s">
+      <c r="S34" s="30"/>
+      <c r="T34" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="T34" s="9"/>
-      <c r="U34" s="20"/>
-      <c r="V34" s="20" t="str">
+      <c r="U34" s="9"/>
+      <c r="V34" s="20"/>
+      <c r="W34" s="20" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="W34" s="20" t="str">
+      <c r="X34" s="20" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="X34" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="35" spans="1:24">
+      <c r="Y34" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="35" spans="1:25">
       <c r="A35" s="6" t="s">
         <v>80</v>
       </c>
@@ -5962,24 +6299,25 @@
         <f t="shared" si="9"/>
         <v/>
       </c>
-      <c r="S35" s="9" t="s">
+      <c r="S35" s="30"/>
+      <c r="T35" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="T35" s="9"/>
-      <c r="U35" s="20"/>
-      <c r="V35" s="20" t="str">
+      <c r="U35" s="9"/>
+      <c r="V35" s="20"/>
+      <c r="W35" s="20" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="W35" s="20" t="str">
+      <c r="X35" s="20" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="X35" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="36" spans="1:24" ht="25.5">
+      <c r="Y35" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="36" spans="1:25" ht="25.5">
       <c r="A36" s="6" t="s">
         <v>80</v>
       </c>
@@ -6028,24 +6366,25 @@
         <f t="shared" si="9"/>
         <v/>
       </c>
-      <c r="S36" s="9" t="s">
+      <c r="S36" s="30"/>
+      <c r="T36" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="T36" s="9"/>
-      <c r="U36" s="20"/>
-      <c r="V36" s="20" t="str">
+      <c r="U36" s="9"/>
+      <c r="V36" s="20"/>
+      <c r="W36" s="20" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="W36" s="20" t="str">
+      <c r="X36" s="20" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="X36" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="37" spans="1:24" ht="25.5">
+      <c r="Y36" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="37" spans="1:25" ht="25.5">
       <c r="A37" s="11" t="s">
         <v>80</v>
       </c>
@@ -6094,29 +6433,39 @@
         <f t="shared" si="9"/>
         <v/>
       </c>
-      <c r="S37" s="14" t="s">
+      <c r="S37" s="30"/>
+      <c r="T37" s="14" t="s">
         <v>58</v>
       </c>
-      <c r="T37" s="14"/>
-      <c r="U37" s="21"/>
-      <c r="V37" s="21" t="str">
+      <c r="U37" s="14"/>
+      <c r="V37" s="21"/>
+      <c r="W37" s="21" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="W37" s="21" t="str">
+      <c r="X37" s="21" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="X37" s="15" t="s">
+      <c r="Y37" s="15" t="s">
         <v>32</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:X1"/>
+    <mergeCell ref="A1:Y1"/>
   </mergeCells>
   <phoneticPr fontId="4" type="noConversion"/>
+  <conditionalFormatting sqref="S4:S23">
+    <cfRule type="expression" dxfId="7" priority="1">
+      <formula>$S4&gt;=$F4</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="6" priority="2">
+      <formula>$S4&lt;$F4</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>